<commit_message>
buscador activo y add product
</commit_message>
<xml_diff>
--- a/docs/Productos.xlsx
+++ b/docs/Productos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Paginas_web\kunanmi\Kunanmi_V1\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8343532-7FA6-4886-8593-D1C0E4A1D79C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832117E1-EEE8-40EA-A9E2-BB4D34F5280F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="2556" windowWidth="17280" windowHeight="8976" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="2" r:id="rId1"/>
@@ -33,8 +33,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -64,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1617" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1617" uniqueCount="553">
   <si>
     <t>ribbon</t>
   </si>
@@ -1785,12 +1783,15 @@
   <si>
     <t>AROMA</t>
   </si>
+  <si>
+    <t>Basic Essences Collection (11)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1863,8 +1864,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1886,6 +1894,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2128,7 +2142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -2210,6 +2224,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2507,12 +2527,13 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="2" max="2" width="25.5546875" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="25.77734375" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" customWidth="1"/>
     <col min="5" max="5" width="15.5546875" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625"/>
-    <col min="8" max="8" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.33203125" customWidth="1"/>
+    <col min="7" max="7" width="7" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="16.33203125" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="12.33203125" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="26" bestFit="1" customWidth="1"/>
@@ -2566,7 +2587,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="2" spans="1:15" hidden="1">
+    <row r="2" spans="1:15" ht="28.8" hidden="1">
       <c r="A2" s="31" t="s">
         <v>476</v>
       </c>
@@ -3174,7 +3195,7 @@
       </c>
       <c r="O20" s="30"/>
     </row>
-    <row r="21" spans="1:15" hidden="1">
+    <row r="21" spans="1:15" ht="43.2" hidden="1">
       <c r="A21" s="31" t="s">
         <v>476</v>
       </c>
@@ -3207,7 +3228,7 @@
       </c>
       <c r="O21" s="30"/>
     </row>
-    <row r="22" spans="1:15" ht="28.8" hidden="1">
+    <row r="22" spans="1:15" ht="43.2" hidden="1">
       <c r="A22" s="31" t="s">
         <v>476</v>
       </c>
@@ -3438,7 +3459,7 @@
       <c r="N28" s="30"/>
       <c r="O28" s="30"/>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" spans="1:15" hidden="1">
       <c r="A29" s="31" t="s">
         <v>475</v>
       </c>
@@ -3467,7 +3488,7 @@
       <c r="N29" s="30"/>
       <c r="O29" s="30"/>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" hidden="1">
       <c r="A30" s="31" t="s">
         <v>475</v>
       </c>
@@ -3502,7 +3523,7 @@
       </c>
       <c r="O30" s="30"/>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" hidden="1">
       <c r="A31" s="31" t="s">
         <v>475</v>
       </c>
@@ -3537,7 +3558,7 @@
       </c>
       <c r="O31" s="30"/>
     </row>
-    <row r="32" spans="1:15">
+    <row r="32" spans="1:15" ht="43.2" hidden="1">
       <c r="A32" s="31" t="s">
         <v>475</v>
       </c>
@@ -3566,7 +3587,7 @@
       <c r="N32" s="30"/>
       <c r="O32" s="30"/>
     </row>
-    <row r="33" spans="1:15">
+    <row r="33" spans="1:15" hidden="1">
       <c r="A33" s="31" t="s">
         <v>475</v>
       </c>
@@ -3597,7 +3618,7 @@
       </c>
       <c r="O33" s="30"/>
     </row>
-    <row r="34" spans="1:15">
+    <row r="34" spans="1:15" hidden="1">
       <c r="A34" s="31" t="s">
         <v>475</v>
       </c>
@@ -3628,7 +3649,7 @@
       </c>
       <c r="O34" s="30"/>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" spans="1:15" hidden="1">
       <c r="A35" s="31" t="s">
         <v>475</v>
       </c>
@@ -3663,7 +3684,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="36" spans="1:15">
+    <row r="36" spans="1:15" hidden="1">
       <c r="A36" s="31" t="s">
         <v>475</v>
       </c>
@@ -3698,7 +3719,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="37" spans="1:15">
+    <row r="37" spans="1:15" hidden="1">
       <c r="A37" s="31" t="s">
         <v>475</v>
       </c>
@@ -3729,7 +3750,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="38" spans="1:15">
+    <row r="38" spans="1:15" hidden="1">
       <c r="A38" s="31" t="s">
         <v>475</v>
       </c>
@@ -3764,7 +3785,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="39" spans="1:15">
+    <row r="39" spans="1:15" hidden="1">
       <c r="A39" s="31" t="s">
         <v>475</v>
       </c>
@@ -3791,7 +3812,7 @@
       <c r="N39" s="30"/>
       <c r="O39" s="30"/>
     </row>
-    <row r="40" spans="1:15">
+    <row r="40" spans="1:15" hidden="1">
       <c r="A40" s="31" t="s">
         <v>475</v>
       </c>
@@ -3818,7 +3839,7 @@
       <c r="N40" s="30"/>
       <c r="O40" s="30"/>
     </row>
-    <row r="41" spans="1:15">
+    <row r="41" spans="1:15" hidden="1">
       <c r="A41" s="31" t="s">
         <v>475</v>
       </c>
@@ -3845,7 +3866,7 @@
       <c r="N41" s="30"/>
       <c r="O41" s="30"/>
     </row>
-    <row r="42" spans="1:15">
+    <row r="42" spans="1:15" hidden="1">
       <c r="A42" s="31" t="s">
         <v>475</v>
       </c>
@@ -3872,7 +3893,7 @@
       <c r="N42" s="30"/>
       <c r="O42" s="30"/>
     </row>
-    <row r="43" spans="1:15">
+    <row r="43" spans="1:15" hidden="1">
       <c r="A43" s="31" t="s">
         <v>475</v>
       </c>
@@ -3899,7 +3920,7 @@
       <c r="N43" s="30"/>
       <c r="O43" s="30"/>
     </row>
-    <row r="44" spans="1:15">
+    <row r="44" spans="1:15" hidden="1">
       <c r="A44" s="31" t="s">
         <v>475</v>
       </c>
@@ -3928,7 +3949,7 @@
       <c r="N44" s="30"/>
       <c r="O44" s="30"/>
     </row>
-    <row r="45" spans="1:15">
+    <row r="45" spans="1:15" hidden="1">
       <c r="A45" s="31" t="s">
         <v>475</v>
       </c>
@@ -3957,7 +3978,7 @@
       <c r="N45" s="30"/>
       <c r="O45" s="30"/>
     </row>
-    <row r="46" spans="1:15">
+    <row r="46" spans="1:15" hidden="1">
       <c r="A46" s="31" t="s">
         <v>475</v>
       </c>
@@ -3986,7 +4007,7 @@
       <c r="N46" s="30"/>
       <c r="O46" s="30"/>
     </row>
-    <row r="47" spans="1:15">
+    <row r="47" spans="1:15" hidden="1">
       <c r="A47" s="31" t="s">
         <v>475</v>
       </c>
@@ -4015,1304 +4036,1304 @@
       <c r="N47" s="30"/>
       <c r="O47" s="30"/>
     </row>
-    <row r="48" spans="1:15" hidden="1">
-      <c r="A48" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B48" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C48" s="30" t="s">
+    <row r="48" spans="1:15" s="53" customFormat="1">
+      <c r="A48" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B48" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C48" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D48" s="30" t="s">
+      <c r="D48" s="52" t="s">
         <v>309</v>
       </c>
       <c r="E48" s="30"/>
-      <c r="F48" s="30">
+      <c r="F48" s="52">
         <v>59</v>
       </c>
-      <c r="G48" s="30">
-        <v>10</v>
-      </c>
-      <c r="H48" s="30"/>
+      <c r="G48" s="52">
+        <v>10</v>
+      </c>
+      <c r="H48" s="52"/>
       <c r="I48" s="30"/>
       <c r="J48" s="30"/>
-      <c r="K48" s="30" t="s">
+      <c r="K48" s="52" t="s">
         <v>309</v>
       </c>
-      <c r="M48" s="30" t="s">
+      <c r="M48" s="52" t="s">
         <v>343</v>
       </c>
-      <c r="N48" s="30"/>
-      <c r="O48" s="30" t="s">
+      <c r="N48" s="52"/>
+      <c r="O48" s="52" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="49" spans="1:15" hidden="1">
-      <c r="A49" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B49" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C49" s="30" t="s">
+    <row r="49" spans="1:15" s="53" customFormat="1">
+      <c r="A49" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B49" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C49" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D49" s="30" t="s">
+      <c r="D49" s="52" t="s">
         <v>367</v>
       </c>
       <c r="E49" s="30"/>
-      <c r="F49" s="30">
+      <c r="F49" s="52">
         <v>59</v>
       </c>
-      <c r="G49" s="30">
-        <v>10</v>
-      </c>
-      <c r="H49" s="30"/>
+      <c r="G49" s="52">
+        <v>10</v>
+      </c>
+      <c r="H49" s="52"/>
       <c r="I49" s="30"/>
       <c r="J49" s="30"/>
-      <c r="K49" s="30" t="s">
+      <c r="K49" s="52" t="s">
         <v>366</v>
       </c>
-      <c r="L49" s="30" t="s">
+      <c r="L49" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="O49" s="30" t="s">
+      <c r="O49" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="50" spans="1:15" hidden="1">
-      <c r="A50" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B50" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C50" s="30" t="s">
+    <row r="50" spans="1:15" s="53" customFormat="1">
+      <c r="A50" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B50" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C50" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D50" s="30" t="s">
+      <c r="D50" s="52" t="s">
         <v>365</v>
       </c>
       <c r="E50" s="30"/>
-      <c r="F50" s="30">
+      <c r="F50" s="52">
         <v>59</v>
       </c>
-      <c r="G50" s="30">
-        <v>10</v>
-      </c>
-      <c r="H50" s="30"/>
+      <c r="G50" s="52">
+        <v>10</v>
+      </c>
+      <c r="H50" s="52"/>
       <c r="I50" s="30"/>
       <c r="J50" s="30"/>
-      <c r="K50" s="30" t="s">
+      <c r="K50" s="52" t="s">
         <v>365</v>
       </c>
-      <c r="L50" s="30" t="s">
+      <c r="L50" s="52" t="s">
         <v>344</v>
       </c>
-      <c r="M50" s="30"/>
-      <c r="N50" s="30"/>
-      <c r="O50" s="30" t="s">
+      <c r="M50" s="52"/>
+      <c r="N50" s="52"/>
+      <c r="O50" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="51" spans="1:15" hidden="1">
-      <c r="A51" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B51" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C51" s="30" t="s">
+    <row r="51" spans="1:15" s="53" customFormat="1">
+      <c r="A51" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B51" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C51" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D51" s="30" t="s">
+      <c r="D51" s="52" t="s">
         <v>347</v>
       </c>
       <c r="E51" s="30"/>
-      <c r="F51" s="30">
+      <c r="F51" s="52">
         <v>59</v>
       </c>
-      <c r="G51" s="30">
-        <v>10</v>
-      </c>
-      <c r="H51" s="30"/>
+      <c r="G51" s="52">
+        <v>10</v>
+      </c>
+      <c r="H51" s="52"/>
       <c r="I51" s="30"/>
       <c r="J51" s="30"/>
-      <c r="K51" s="30" t="s">
+      <c r="K51" s="52" t="s">
         <v>347</v>
       </c>
-      <c r="L51" s="30"/>
-      <c r="M51" s="30" t="s">
+      <c r="L51" s="52"/>
+      <c r="M51" s="54" t="s">
         <v>348</v>
       </c>
-      <c r="N51" s="30"/>
-      <c r="O51" s="30" t="s">
+      <c r="N51" s="52"/>
+      <c r="O51" s="54" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="52" spans="1:15" hidden="1">
-      <c r="A52" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B52" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C52" s="30" t="s">
+    <row r="52" spans="1:15" s="53" customFormat="1">
+      <c r="A52" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B52" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C52" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D52" s="30" t="s">
+      <c r="D52" s="52" t="s">
         <v>340</v>
       </c>
       <c r="E52" s="30"/>
-      <c r="F52" s="30">
+      <c r="F52" s="52">
         <v>59</v>
       </c>
-      <c r="G52" s="30">
-        <v>10</v>
-      </c>
-      <c r="H52" s="30"/>
+      <c r="G52" s="52">
+        <v>10</v>
+      </c>
+      <c r="H52" s="52"/>
       <c r="I52" s="30"/>
       <c r="J52" s="30"/>
-      <c r="K52" s="30" t="s">
+      <c r="K52" s="52" t="s">
         <v>340</v>
       </c>
-      <c r="L52" s="30" t="s">
+      <c r="L52" s="54" t="s">
         <v>344</v>
       </c>
-      <c r="M52" s="30" t="s">
+      <c r="M52" s="54" t="s">
         <v>348</v>
       </c>
-      <c r="N52" s="30"/>
-      <c r="O52" s="30" t="s">
+      <c r="N52" s="52"/>
+      <c r="O52" s="54" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="53" spans="1:15" hidden="1">
-      <c r="A53" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B53" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C53" s="30" t="s">
+    <row r="53" spans="1:15" s="53" customFormat="1">
+      <c r="A53" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B53" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C53" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D53" s="30" t="s">
+      <c r="D53" s="52" t="s">
         <v>310</v>
       </c>
       <c r="E53" s="30"/>
-      <c r="F53" s="30">
+      <c r="F53" s="52">
         <v>59</v>
       </c>
-      <c r="G53" s="30">
-        <v>10</v>
-      </c>
-      <c r="H53" s="30"/>
+      <c r="G53" s="52">
+        <v>10</v>
+      </c>
+      <c r="H53" s="52"/>
       <c r="I53" s="30"/>
       <c r="J53" s="30"/>
-      <c r="K53" s="30" t="s">
+      <c r="K53" s="52" t="s">
         <v>310</v>
       </c>
-      <c r="L53" s="30"/>
-      <c r="M53" s="30" t="s">
+      <c r="L53" s="52"/>
+      <c r="M53" s="54" t="s">
         <v>348</v>
       </c>
-      <c r="N53" s="30"/>
-      <c r="O53" s="30" t="s">
+      <c r="N53" s="52"/>
+      <c r="O53" s="54" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="54" spans="1:15" hidden="1">
-      <c r="A54" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B54" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C54" s="30" t="s">
+    <row r="54" spans="1:15" s="53" customFormat="1">
+      <c r="A54" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B54" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C54" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D54" s="30" t="s">
+      <c r="D54" s="52" t="s">
         <v>311</v>
       </c>
       <c r="E54" s="30"/>
-      <c r="F54" s="30">
+      <c r="F54" s="52">
         <v>59</v>
       </c>
-      <c r="G54" s="30">
-        <v>10</v>
-      </c>
-      <c r="H54" s="30"/>
+      <c r="G54" s="52">
+        <v>10</v>
+      </c>
+      <c r="H54" s="52"/>
       <c r="I54" s="30"/>
       <c r="J54" s="30"/>
-      <c r="K54" s="30" t="s">
+      <c r="K54" s="52" t="s">
         <v>311</v>
       </c>
-      <c r="L54" s="30"/>
-      <c r="M54" s="30" t="s">
+      <c r="L54" s="52"/>
+      <c r="M54" s="54" t="s">
         <v>348</v>
       </c>
-      <c r="N54" s="30"/>
-      <c r="O54" s="30" t="s">
+      <c r="N54" s="52"/>
+      <c r="O54" s="54" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="55" spans="1:15" hidden="1">
-      <c r="A55" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B55" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C55" s="30" t="s">
+    <row r="55" spans="1:15" s="53" customFormat="1">
+      <c r="A55" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B55" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C55" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D55" s="30" t="s">
+      <c r="D55" s="52" t="s">
         <v>312</v>
       </c>
       <c r="E55" s="30"/>
-      <c r="F55" s="30">
+      <c r="F55" s="52">
         <v>59</v>
       </c>
-      <c r="G55" s="30">
-        <v>10</v>
-      </c>
-      <c r="H55" s="30"/>
+      <c r="G55" s="52">
+        <v>10</v>
+      </c>
+      <c r="H55" s="52"/>
       <c r="I55" s="30"/>
       <c r="J55" s="30"/>
-      <c r="K55" s="30" t="s">
+      <c r="K55" s="52" t="s">
         <v>312</v>
       </c>
-      <c r="L55" s="30"/>
-      <c r="M55" s="30" t="s">
+      <c r="L55" s="52"/>
+      <c r="M55" s="54" t="s">
         <v>348</v>
       </c>
-      <c r="N55" s="30"/>
-      <c r="O55" s="30" t="s">
+      <c r="N55" s="52"/>
+      <c r="O55" s="54" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="56" spans="1:15" hidden="1">
-      <c r="A56" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B56" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C56" s="30" t="s">
+    <row r="56" spans="1:15" s="53" customFormat="1">
+      <c r="A56" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B56" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C56" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D56" s="30" t="s">
+      <c r="D56" s="52" t="s">
         <v>313</v>
       </c>
       <c r="E56" s="30"/>
-      <c r="F56" s="30">
+      <c r="F56" s="52">
         <v>59</v>
       </c>
-      <c r="G56" s="30">
+      <c r="G56" s="52">
         <v>10</v>
       </c>
       <c r="H56" s="30"/>
       <c r="I56" s="30"/>
       <c r="J56" s="30"/>
-      <c r="K56" s="30" t="s">
+      <c r="K56" s="52" t="s">
         <v>313</v>
       </c>
-      <c r="L56" s="30" t="s">
+      <c r="L56" s="52" t="s">
         <v>344</v>
       </c>
-      <c r="M56" s="30" t="s">
+      <c r="M56" s="54" t="s">
         <v>348</v>
       </c>
-      <c r="N56" s="30"/>
-      <c r="O56" s="30" t="s">
+      <c r="N56" s="52"/>
+      <c r="O56" s="54" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="57" spans="1:15" hidden="1">
-      <c r="A57" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B57" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C57" s="30" t="s">
+    <row r="57" spans="1:15" s="53" customFormat="1">
+      <c r="A57" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B57" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C57" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D57" s="30" t="s">
+      <c r="D57" s="52" t="s">
         <v>314</v>
       </c>
       <c r="E57" s="30"/>
-      <c r="F57" s="30">
+      <c r="F57" s="52">
         <v>59</v>
       </c>
-      <c r="G57" s="30">
+      <c r="G57" s="52">
         <v>10</v>
       </c>
       <c r="H57" s="30"/>
       <c r="I57" s="30"/>
       <c r="J57" s="30"/>
-      <c r="K57" s="30" t="s">
+      <c r="K57" s="52" t="s">
         <v>314</v>
       </c>
-      <c r="L57" s="30"/>
-      <c r="M57" s="30" t="s">
+      <c r="L57" s="52"/>
+      <c r="M57" s="52" t="s">
         <v>343</v>
       </c>
-      <c r="N57" s="30"/>
-      <c r="O57" s="30"/>
-    </row>
-    <row r="58" spans="1:15" hidden="1">
-      <c r="A58" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B58" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C58" s="30" t="s">
+      <c r="N57" s="52"/>
+      <c r="O57" s="52"/>
+    </row>
+    <row r="58" spans="1:15" s="53" customFormat="1">
+      <c r="A58" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B58" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C58" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D58" s="30" t="s">
+      <c r="D58" s="52" t="s">
         <v>315</v>
       </c>
       <c r="E58" s="30"/>
-      <c r="F58" s="30">
+      <c r="F58" s="52">
         <v>59</v>
       </c>
-      <c r="G58" s="30">
+      <c r="G58" s="52">
         <v>10</v>
       </c>
       <c r="H58" s="30"/>
       <c r="I58" s="30"/>
       <c r="J58" s="30"/>
-      <c r="K58" s="30" t="s">
+      <c r="K58" s="52" t="s">
         <v>315</v>
       </c>
-      <c r="L58" s="30"/>
-      <c r="M58" s="30" t="s">
+      <c r="L58" s="52"/>
+      <c r="M58" s="52" t="s">
         <v>343</v>
       </c>
-      <c r="N58" s="30"/>
-      <c r="O58" s="30"/>
-    </row>
-    <row r="59" spans="1:15" hidden="1">
-      <c r="A59" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B59" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C59" s="30" t="s">
+      <c r="N58" s="52"/>
+      <c r="O58" s="52"/>
+    </row>
+    <row r="59" spans="1:15" s="53" customFormat="1">
+      <c r="A59" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B59" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C59" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D59" s="30" t="s">
+      <c r="D59" s="52" t="s">
         <v>316</v>
       </c>
       <c r="E59" s="30"/>
-      <c r="F59" s="30">
+      <c r="F59" s="52">
         <v>59</v>
       </c>
-      <c r="G59" s="30">
+      <c r="G59" s="52">
         <v>10</v>
       </c>
       <c r="H59" s="30"/>
       <c r="I59" s="30"/>
       <c r="J59" s="30"/>
-      <c r="K59" s="30" t="s">
+      <c r="K59" s="52" t="s">
         <v>316</v>
       </c>
-      <c r="L59" s="30"/>
-      <c r="M59" s="30" t="s">
+      <c r="L59" s="52"/>
+      <c r="M59" s="52" t="s">
         <v>343</v>
       </c>
-      <c r="N59" s="30"/>
-      <c r="O59" s="30"/>
-    </row>
-    <row r="60" spans="1:15" hidden="1">
-      <c r="A60" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B60" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C60" s="30" t="s">
+      <c r="N59" s="52"/>
+      <c r="O59" s="52"/>
+    </row>
+    <row r="60" spans="1:15" s="53" customFormat="1">
+      <c r="A60" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B60" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C60" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D60" s="30" t="s">
+      <c r="D60" s="52" t="s">
         <v>363</v>
       </c>
       <c r="E60" s="30"/>
-      <c r="F60" s="30">
+      <c r="F60" s="52">
         <v>59</v>
       </c>
-      <c r="G60" s="30">
+      <c r="G60" s="52">
         <v>10</v>
       </c>
       <c r="H60" s="30"/>
       <c r="I60" s="30"/>
       <c r="J60" s="30"/>
-      <c r="K60" s="30" t="s">
+      <c r="K60" s="52" t="s">
         <v>317</v>
       </c>
-      <c r="L60" s="30"/>
-      <c r="M60" s="30" t="s">
+      <c r="L60" s="52"/>
+      <c r="M60" s="52" t="s">
         <v>343</v>
       </c>
-      <c r="N60" s="30"/>
-      <c r="O60" s="30" t="s">
+      <c r="N60" s="52"/>
+      <c r="O60" s="52" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="61" spans="1:15" hidden="1">
-      <c r="A61" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B61" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C61" s="30" t="s">
+    <row r="61" spans="1:15" s="53" customFormat="1">
+      <c r="A61" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B61" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C61" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D61" s="30" t="s">
+      <c r="D61" s="52" t="s">
         <v>318</v>
       </c>
       <c r="E61" s="30"/>
-      <c r="F61" s="30">
+      <c r="F61" s="52">
         <v>59</v>
       </c>
-      <c r="G61" s="30">
+      <c r="G61" s="52">
         <v>10</v>
       </c>
       <c r="H61" s="30"/>
       <c r="I61" s="30"/>
       <c r="J61" s="30"/>
-      <c r="K61" s="30" t="s">
+      <c r="K61" s="52" t="s">
         <v>318</v>
       </c>
-      <c r="L61" s="30" t="s">
+      <c r="L61" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M61" s="30" t="s">
+      <c r="M61" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N61" s="30"/>
-      <c r="O61" s="30" t="s">
+      <c r="N61" s="52"/>
+      <c r="O61" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="62" spans="1:15" hidden="1">
-      <c r="A62" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B62" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C62" s="30" t="s">
+    <row r="62" spans="1:15" s="53" customFormat="1">
+      <c r="A62" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B62" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C62" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D62" s="30" t="s">
+      <c r="D62" s="52" t="s">
         <v>339</v>
       </c>
       <c r="E62" s="30"/>
-      <c r="F62" s="30">
+      <c r="F62" s="52">
         <v>59</v>
       </c>
-      <c r="G62" s="30">
+      <c r="G62" s="52">
         <v>10</v>
       </c>
       <c r="H62" s="30"/>
       <c r="I62" s="30"/>
       <c r="J62" s="30"/>
-      <c r="K62" s="30" t="s">
+      <c r="K62" s="52" t="s">
         <v>339</v>
       </c>
-      <c r="L62" s="30" t="s">
+      <c r="L62" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M62" s="30" t="s">
+      <c r="M62" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N62" s="30"/>
-      <c r="O62" s="30" t="s">
+      <c r="N62" s="52"/>
+      <c r="O62" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="63" spans="1:15" hidden="1">
-      <c r="A63" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B63" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C63" s="30" t="s">
+    <row r="63" spans="1:15" s="53" customFormat="1">
+      <c r="A63" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B63" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C63" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D63" s="30" t="s">
+      <c r="D63" s="52" t="s">
         <v>319</v>
       </c>
       <c r="E63" s="30"/>
-      <c r="F63" s="30">
+      <c r="F63" s="52">
         <v>59</v>
       </c>
-      <c r="G63" s="30">
+      <c r="G63" s="52">
         <v>10</v>
       </c>
       <c r="H63" s="30"/>
       <c r="I63" s="30"/>
       <c r="J63" s="30"/>
-      <c r="K63" s="30" t="s">
+      <c r="K63" s="52" t="s">
         <v>319</v>
       </c>
-      <c r="L63" s="30" t="s">
+      <c r="L63" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M63" s="30" t="s">
+      <c r="M63" s="52" t="s">
         <v>349</v>
       </c>
-      <c r="N63" s="30"/>
-      <c r="O63" s="30" t="s">
+      <c r="N63" s="52"/>
+      <c r="O63" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="64" spans="1:15" hidden="1">
-      <c r="A64" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B64" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C64" s="30" t="s">
+    <row r="64" spans="1:15" s="53" customFormat="1">
+      <c r="A64" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B64" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C64" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D64" s="30" t="s">
+      <c r="D64" s="52" t="s">
         <v>320</v>
       </c>
       <c r="E64" s="30"/>
-      <c r="F64" s="30">
+      <c r="F64" s="52">
         <v>59</v>
       </c>
-      <c r="G64" s="30">
+      <c r="G64" s="52">
         <v>10</v>
       </c>
       <c r="H64" s="30"/>
       <c r="I64" s="30"/>
       <c r="J64" s="30"/>
-      <c r="K64" s="30" t="s">
+      <c r="K64" s="52" t="s">
         <v>320</v>
       </c>
-      <c r="L64" s="30" t="s">
+      <c r="L64" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M64" s="30" t="s">
+      <c r="M64" s="52" t="s">
         <v>349</v>
       </c>
-      <c r="N64" s="30"/>
-      <c r="O64" s="30" t="s">
+      <c r="N64" s="52"/>
+      <c r="O64" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="65" spans="1:15" hidden="1">
-      <c r="A65" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B65" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C65" s="30" t="s">
+    <row r="65" spans="1:15" s="53" customFormat="1">
+      <c r="A65" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B65" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C65" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D65" s="30" t="s">
+      <c r="D65" s="52" t="s">
         <v>321</v>
       </c>
       <c r="E65" s="30"/>
-      <c r="F65" s="30">
+      <c r="F65" s="52">
         <v>59</v>
       </c>
-      <c r="G65" s="30">
+      <c r="G65" s="52">
         <v>10</v>
       </c>
       <c r="H65" s="30"/>
       <c r="I65" s="30"/>
       <c r="J65" s="30"/>
-      <c r="K65" s="30" t="s">
+      <c r="K65" s="52" t="s">
         <v>321</v>
       </c>
-      <c r="L65" s="30" t="s">
+      <c r="L65" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M65" s="30" t="s">
+      <c r="M65" s="52" t="s">
         <v>349</v>
       </c>
-      <c r="N65" s="30"/>
-      <c r="O65" s="30" t="s">
+      <c r="N65" s="52"/>
+      <c r="O65" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="66" spans="1:15" hidden="1">
-      <c r="A66" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B66" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C66" s="30" t="s">
+    <row r="66" spans="1:15" s="53" customFormat="1">
+      <c r="A66" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B66" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C66" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D66" s="30" t="s">
+      <c r="D66" s="52" t="s">
         <v>322</v>
       </c>
       <c r="E66" s="30"/>
-      <c r="F66" s="30">
+      <c r="F66" s="52">
         <v>59</v>
       </c>
-      <c r="G66" s="30">
+      <c r="G66" s="52">
         <v>10</v>
       </c>
       <c r="H66" s="30"/>
       <c r="I66" s="30"/>
       <c r="J66" s="30"/>
-      <c r="K66" s="30" t="s">
+      <c r="K66" s="52" t="s">
         <v>322</v>
       </c>
-      <c r="L66" s="30" t="s">
+      <c r="L66" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M66" s="30" t="s">
+      <c r="M66" s="52" t="s">
         <v>349</v>
       </c>
-      <c r="N66" s="30"/>
-      <c r="O66" s="30" t="s">
+      <c r="N66" s="52"/>
+      <c r="O66" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="67" spans="1:15" hidden="1">
-      <c r="A67" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B67" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C67" s="30" t="s">
-        <v>341</v>
-      </c>
-      <c r="D67" s="30" t="s">
+    <row r="67" spans="1:15" s="53" customFormat="1">
+      <c r="A67" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B67" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C67" s="52" t="s">
+        <v>552</v>
+      </c>
+      <c r="D67" s="52" t="s">
         <v>324</v>
       </c>
       <c r="E67" s="30"/>
-      <c r="F67" s="30">
+      <c r="F67" s="52">
         <v>59</v>
       </c>
-      <c r="G67" s="30">
+      <c r="G67" s="52">
         <v>10</v>
       </c>
       <c r="H67" s="30"/>
       <c r="I67" s="30"/>
       <c r="J67" s="30"/>
-      <c r="K67" s="30" t="s">
+      <c r="K67" s="52" t="s">
         <v>324</v>
       </c>
-      <c r="L67" s="30" t="s">
+      <c r="L67" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M67" s="30" t="s">
+      <c r="M67" s="52" t="s">
         <v>349</v>
       </c>
-      <c r="N67" s="30"/>
-      <c r="O67" s="30" t="s">
+      <c r="N67" s="52"/>
+      <c r="O67" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="68" spans="1:15" hidden="1">
-      <c r="A68" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B68" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C68" s="30" t="s">
+    <row r="68" spans="1:15" s="53" customFormat="1">
+      <c r="A68" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B68" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C68" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D68" s="30" t="s">
+      <c r="D68" s="52" t="s">
         <v>323</v>
       </c>
       <c r="E68" s="30"/>
-      <c r="F68" s="30">
+      <c r="F68" s="52">
         <v>59</v>
       </c>
-      <c r="G68" s="30">
+      <c r="G68" s="52">
         <v>10</v>
       </c>
       <c r="H68" s="30"/>
       <c r="I68" s="30"/>
       <c r="J68" s="30"/>
-      <c r="K68" s="30" t="s">
+      <c r="K68" s="52" t="s">
         <v>323</v>
       </c>
-      <c r="L68" s="30" t="s">
+      <c r="L68" s="52" t="s">
         <v>343</v>
       </c>
-      <c r="M68" s="30" t="s">
+      <c r="M68" s="52" t="s">
         <v>349</v>
       </c>
-      <c r="N68" s="30"/>
-      <c r="O68" s="30" t="s">
+      <c r="N68" s="52"/>
+      <c r="O68" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="69" spans="1:15" hidden="1">
-      <c r="A69" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B69" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C69" s="30" t="s">
+    <row r="69" spans="1:15" s="53" customFormat="1">
+      <c r="A69" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B69" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C69" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D69" s="30" t="s">
+      <c r="D69" s="52" t="s">
         <v>325</v>
       </c>
       <c r="E69" s="30"/>
-      <c r="F69" s="30">
+      <c r="F69" s="52">
         <v>59</v>
       </c>
-      <c r="G69" s="30">
+      <c r="G69" s="52">
         <v>10</v>
       </c>
       <c r="H69" s="30"/>
       <c r="I69" s="30"/>
       <c r="J69" s="30"/>
-      <c r="K69" s="30" t="s">
+      <c r="K69" s="52" t="s">
         <v>325</v>
       </c>
-      <c r="L69" s="30" t="s">
+      <c r="L69" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M69" s="30" t="s">
+      <c r="M69" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N69" s="30"/>
-      <c r="O69" s="30" t="s">
+      <c r="N69" s="52"/>
+      <c r="O69" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="70" spans="1:15" hidden="1">
-      <c r="A70" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B70" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C70" s="30" t="s">
+    <row r="70" spans="1:15" s="53" customFormat="1">
+      <c r="A70" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B70" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C70" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D70" s="30" t="s">
+      <c r="D70" s="52" t="s">
         <v>326</v>
       </c>
       <c r="E70" s="30"/>
-      <c r="F70" s="30">
+      <c r="F70" s="52">
         <v>59</v>
       </c>
-      <c r="G70" s="30">
+      <c r="G70" s="52">
         <v>10</v>
       </c>
       <c r="H70" s="30"/>
       <c r="I70" s="30"/>
       <c r="J70" s="30"/>
-      <c r="K70" s="30" t="s">
+      <c r="K70" s="52" t="s">
         <v>326</v>
       </c>
-      <c r="L70" s="30" t="s">
+      <c r="L70" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M70" s="30" t="s">
+      <c r="M70" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N70" s="30"/>
-      <c r="O70" s="30" t="s">
+      <c r="N70" s="52"/>
+      <c r="O70" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="71" spans="1:15" hidden="1">
-      <c r="A71" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B71" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C71" s="30" t="s">
+    <row r="71" spans="1:15" s="53" customFormat="1">
+      <c r="A71" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B71" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C71" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D71" s="30" t="s">
+      <c r="D71" s="52" t="s">
         <v>327</v>
       </c>
       <c r="E71" s="30"/>
-      <c r="F71" s="30">
+      <c r="F71" s="52">
         <v>59</v>
       </c>
-      <c r="G71" s="30">
+      <c r="G71" s="52">
         <v>10</v>
       </c>
       <c r="H71" s="30"/>
       <c r="I71" s="30"/>
       <c r="J71" s="30"/>
-      <c r="K71" s="30" t="s">
+      <c r="K71" s="52" t="s">
         <v>327</v>
       </c>
-      <c r="L71" s="30" t="s">
+      <c r="L71" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M71" s="30" t="s">
+      <c r="M71" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N71" s="30"/>
-      <c r="O71" s="30" t="s">
+      <c r="N71" s="52"/>
+      <c r="O71" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="72" spans="1:15" hidden="1">
-      <c r="A72" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B72" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C72" s="30" t="s">
+    <row r="72" spans="1:15" s="53" customFormat="1">
+      <c r="A72" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B72" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C72" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D72" s="30" t="s">
+      <c r="D72" s="52" t="s">
         <v>328</v>
       </c>
       <c r="E72" s="30"/>
-      <c r="F72" s="30">
+      <c r="F72" s="52">
         <v>59</v>
       </c>
-      <c r="G72" s="30">
+      <c r="G72" s="52">
         <v>10</v>
       </c>
       <c r="H72" s="30"/>
       <c r="I72" s="30"/>
       <c r="J72" s="30"/>
-      <c r="K72" s="30" t="s">
+      <c r="K72" s="52" t="s">
         <v>328</v>
       </c>
-      <c r="L72" s="30" t="s">
+      <c r="L72" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M72" s="30" t="s">
+      <c r="M72" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N72" s="30"/>
-      <c r="O72" s="30" t="s">
+      <c r="N72" s="52"/>
+      <c r="O72" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="73" spans="1:15" hidden="1">
-      <c r="A73" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B73" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C73" s="30" t="s">
+    <row r="73" spans="1:15" s="53" customFormat="1">
+      <c r="A73" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B73" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C73" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D73" s="30" t="s">
+      <c r="D73" s="52" t="s">
         <v>329</v>
       </c>
       <c r="E73" s="30"/>
-      <c r="F73" s="30">
+      <c r="F73" s="52">
         <v>59</v>
       </c>
-      <c r="G73" s="30">
+      <c r="G73" s="52">
         <v>10</v>
       </c>
       <c r="H73" s="30"/>
       <c r="I73" s="30"/>
       <c r="J73" s="30"/>
-      <c r="K73" s="30" t="s">
+      <c r="K73" s="52" t="s">
         <v>329</v>
       </c>
-      <c r="L73" s="30" t="s">
+      <c r="L73" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M73" s="30" t="s">
+      <c r="M73" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N73" s="30"/>
-      <c r="O73" s="30" t="s">
+      <c r="N73" s="52"/>
+      <c r="O73" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="74" spans="1:15" hidden="1">
-      <c r="A74" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B74" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C74" s="30" t="s">
+    <row r="74" spans="1:15" s="53" customFormat="1">
+      <c r="A74" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B74" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C74" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D74" s="30" t="s">
+      <c r="D74" s="52" t="s">
         <v>330</v>
       </c>
       <c r="E74" s="30"/>
-      <c r="F74" s="30">
+      <c r="F74" s="52">
         <v>59</v>
       </c>
-      <c r="G74" s="30">
+      <c r="G74" s="52">
         <v>10</v>
       </c>
       <c r="H74" s="30"/>
       <c r="I74" s="30"/>
       <c r="J74" s="30"/>
-      <c r="K74" s="30" t="s">
+      <c r="K74" s="52" t="s">
         <v>330</v>
       </c>
-      <c r="L74" s="30" t="s">
+      <c r="L74" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M74" s="30" t="s">
+      <c r="M74" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N74" s="30"/>
-      <c r="O74" s="30" t="s">
+      <c r="N74" s="52"/>
+      <c r="O74" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="75" spans="1:15" hidden="1">
-      <c r="A75" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B75" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C75" s="30" t="s">
+    <row r="75" spans="1:15" s="53" customFormat="1">
+      <c r="A75" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B75" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C75" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D75" s="30" t="s">
+      <c r="D75" s="52" t="s">
         <v>331</v>
       </c>
       <c r="E75" s="30"/>
-      <c r="F75" s="30">
+      <c r="F75" s="52">
         <v>59</v>
       </c>
-      <c r="G75" s="30">
+      <c r="G75" s="52">
         <v>10</v>
       </c>
       <c r="H75" s="30"/>
       <c r="I75" s="30"/>
       <c r="J75" s="30"/>
-      <c r="K75" s="30" t="s">
+      <c r="K75" s="52" t="s">
         <v>331</v>
       </c>
-      <c r="L75" s="30" t="s">
+      <c r="L75" s="52" t="s">
         <v>344</v>
       </c>
-      <c r="M75" s="30"/>
-      <c r="N75" s="30"/>
-      <c r="O75" s="30" t="s">
+      <c r="M75" s="52"/>
+      <c r="N75" s="52"/>
+      <c r="O75" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="76" spans="1:15" hidden="1">
-      <c r="A76" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B76" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C76" s="30" t="s">
+    <row r="76" spans="1:15" s="53" customFormat="1">
+      <c r="A76" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B76" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C76" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D76" s="30" t="s">
+      <c r="D76" s="52" t="s">
         <v>332</v>
       </c>
       <c r="E76" s="30"/>
-      <c r="F76" s="30">
+      <c r="F76" s="52">
         <v>59</v>
       </c>
-      <c r="G76" s="30">
+      <c r="G76" s="52">
         <v>10</v>
       </c>
       <c r="H76" s="30"/>
       <c r="I76" s="30"/>
       <c r="J76" s="30"/>
-      <c r="K76" s="30" t="s">
+      <c r="K76" s="52" t="s">
         <v>332</v>
       </c>
-      <c r="L76" s="30" t="s">
+      <c r="L76" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M76" s="30" t="s">
+      <c r="M76" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N76" s="30"/>
-      <c r="O76" s="30" t="s">
+      <c r="N76" s="52"/>
+      <c r="O76" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="77" spans="1:15" hidden="1">
-      <c r="A77" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B77" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C77" s="30" t="s">
+    <row r="77" spans="1:15" s="53" customFormat="1">
+      <c r="A77" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B77" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C77" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D77" s="30" t="s">
+      <c r="D77" s="52" t="s">
         <v>333</v>
       </c>
       <c r="E77" s="30"/>
-      <c r="F77" s="30">
+      <c r="F77" s="52">
         <v>59</v>
       </c>
-      <c r="G77" s="30">
+      <c r="G77" s="52">
         <v>10</v>
       </c>
       <c r="H77" s="30"/>
       <c r="I77" s="30"/>
       <c r="J77" s="30"/>
-      <c r="K77" s="30" t="s">
+      <c r="K77" s="52" t="s">
         <v>333</v>
       </c>
-      <c r="L77" s="30"/>
-      <c r="M77" s="30" t="s">
+      <c r="L77" s="52"/>
+      <c r="M77" s="52" t="s">
         <v>350</v>
       </c>
-      <c r="N77" s="30"/>
-      <c r="O77" s="30" t="s">
+      <c r="N77" s="52"/>
+      <c r="O77" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="78" spans="1:15" hidden="1">
-      <c r="A78" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B78" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C78" s="30" t="s">
+    <row r="78" spans="1:15" s="53" customFormat="1">
+      <c r="A78" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B78" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C78" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D78" s="30" t="s">
+      <c r="D78" s="52" t="s">
         <v>334</v>
       </c>
       <c r="E78" s="30"/>
-      <c r="F78" s="30">
+      <c r="F78" s="52">
         <v>59</v>
       </c>
-      <c r="G78" s="30">
+      <c r="G78" s="52">
         <v>10</v>
       </c>
       <c r="H78" s="30"/>
       <c r="I78" s="30"/>
       <c r="J78" s="30"/>
-      <c r="K78" s="30" t="s">
+      <c r="K78" s="52" t="s">
         <v>334</v>
       </c>
-      <c r="L78" s="30" t="s">
+      <c r="L78" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M78" s="30" t="s">
+      <c r="M78" s="52" t="s">
         <v>460</v>
       </c>
-      <c r="N78" s="30"/>
-      <c r="O78" s="30" t="s">
+      <c r="N78" s="52"/>
+      <c r="O78" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="79" spans="1:15" hidden="1">
-      <c r="A79" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B79" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C79" s="30" t="s">
+    <row r="79" spans="1:15" s="53" customFormat="1">
+      <c r="A79" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B79" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C79" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D79" s="30" t="s">
+      <c r="D79" s="52" t="s">
         <v>335</v>
       </c>
       <c r="E79" s="30"/>
-      <c r="F79" s="30">
+      <c r="F79" s="52">
         <v>59</v>
       </c>
-      <c r="G79" s="30">
+      <c r="G79" s="52">
         <v>10</v>
       </c>
       <c r="H79" s="30"/>
       <c r="I79" s="30"/>
       <c r="J79" s="30"/>
-      <c r="K79" s="30" t="s">
+      <c r="K79" s="52" t="s">
         <v>335</v>
       </c>
-      <c r="L79" s="30" t="s">
+      <c r="L79" s="52" t="s">
         <v>346</v>
       </c>
-      <c r="M79" s="30" t="s">
+      <c r="M79" s="52" t="s">
         <v>460</v>
       </c>
-      <c r="N79" s="30"/>
-      <c r="O79" s="30" t="s">
+      <c r="N79" s="52"/>
+      <c r="O79" s="52" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="80" spans="1:15" hidden="1">
-      <c r="A80" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B80" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C80" s="30" t="s">
+    <row r="80" spans="1:15" s="53" customFormat="1">
+      <c r="A80" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B80" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C80" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D80" s="30" t="s">
+      <c r="D80" s="52" t="s">
         <v>336</v>
       </c>
       <c r="E80" s="30"/>
-      <c r="F80" s="30">
+      <c r="F80" s="52">
         <v>59</v>
       </c>
-      <c r="G80" s="30">
+      <c r="G80" s="52">
         <v>10</v>
       </c>
       <c r="H80" s="30"/>
       <c r="I80" s="30"/>
       <c r="J80" s="30"/>
-      <c r="K80" s="30" t="s">
+      <c r="K80" s="52" t="s">
         <v>336</v>
       </c>
-      <c r="L80" s="30" t="s">
+      <c r="L80" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M80" s="30" t="s">
+      <c r="M80" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N80" s="30"/>
-      <c r="O80" s="30" t="s">
+      <c r="N80" s="52"/>
+      <c r="O80" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="81" spans="1:15" hidden="1">
-      <c r="A81" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B81" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C81" s="30" t="s">
+    <row r="81" spans="1:15" s="53" customFormat="1">
+      <c r="A81" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B81" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C81" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D81" s="30" t="s">
+      <c r="D81" s="52" t="s">
         <v>337</v>
       </c>
       <c r="E81" s="30"/>
-      <c r="F81" s="30">
+      <c r="F81" s="52">
         <v>59</v>
       </c>
-      <c r="G81" s="30">
+      <c r="G81" s="52">
         <v>10</v>
       </c>
       <c r="H81" s="30"/>
       <c r="I81" s="30"/>
       <c r="J81" s="30"/>
-      <c r="K81" s="30" t="s">
+      <c r="K81" s="52" t="s">
         <v>337</v>
       </c>
-      <c r="L81" s="30" t="s">
+      <c r="L81" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M81" s="30" t="s">
+      <c r="M81" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N81" s="30"/>
-      <c r="O81" s="30" t="s">
+      <c r="N81" s="52"/>
+      <c r="O81" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="82" spans="1:15" hidden="1">
-      <c r="A82" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B82" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C82" s="30" t="s">
+    <row r="82" spans="1:15" s="53" customFormat="1">
+      <c r="A82" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B82" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C82" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D82" s="30" t="s">
+      <c r="D82" s="52" t="s">
         <v>364</v>
       </c>
       <c r="E82" s="30"/>
-      <c r="F82" s="30">
+      <c r="F82" s="52">
         <v>59</v>
       </c>
-      <c r="G82" s="30">
+      <c r="G82" s="52">
         <v>10</v>
       </c>
       <c r="H82" s="30"/>
       <c r="I82" s="30"/>
       <c r="J82" s="30"/>
-      <c r="K82" s="30" t="s">
+      <c r="K82" s="52" t="s">
         <v>364</v>
       </c>
-      <c r="L82" s="30" t="s">
+      <c r="L82" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M82" s="30" t="s">
+      <c r="M82" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N82" s="30"/>
-      <c r="O82" s="30" t="s">
+      <c r="N82" s="52"/>
+      <c r="O82" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="83" spans="1:15" hidden="1">
-      <c r="A83" s="31" t="s">
-        <v>477</v>
-      </c>
-      <c r="B83" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="C83" s="30" t="s">
+    <row r="83" spans="1:15" s="53" customFormat="1">
+      <c r="A83" s="51" t="s">
+        <v>477</v>
+      </c>
+      <c r="B83" s="52" t="s">
+        <v>493</v>
+      </c>
+      <c r="C83" s="52" t="s">
         <v>341</v>
       </c>
-      <c r="D83" s="30" t="s">
+      <c r="D83" s="52" t="s">
         <v>338</v>
       </c>
       <c r="E83" s="30"/>
-      <c r="F83" s="30">
+      <c r="F83" s="52">
         <v>59</v>
       </c>
-      <c r="G83" s="30">
+      <c r="G83" s="52">
         <v>10</v>
       </c>
       <c r="H83" s="30"/>
       <c r="I83" s="30"/>
       <c r="J83" s="30"/>
-      <c r="K83" s="30" t="s">
+      <c r="K83" s="52" t="s">
         <v>338</v>
       </c>
-      <c r="L83" s="30" t="s">
+      <c r="L83" s="52" t="s">
         <v>345</v>
       </c>
-      <c r="M83" s="30" t="s">
+      <c r="M83" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="N83" s="30"/>
-      <c r="O83" s="30" t="s">
+      <c r="N83" s="52"/>
+      <c r="O83" s="52" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="84" spans="1:15" hidden="1">
+    <row r="84" spans="1:15">
       <c r="A84" s="31" t="s">
         <v>477</v>
       </c>
@@ -5345,7 +5366,7 @@
       <c r="N84" s="30"/>
       <c r="O84" s="30"/>
     </row>
-    <row r="85" spans="1:15" hidden="1">
+    <row r="85" spans="1:15">
       <c r="A85" s="31" t="s">
         <v>477</v>
       </c>
@@ -5378,7 +5399,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="86" spans="1:15" hidden="1">
+    <row r="86" spans="1:15">
       <c r="A86" s="31" t="s">
         <v>477</v>
       </c>
@@ -5411,7 +5432,7 @@
       <c r="N86" s="30"/>
       <c r="O86" s="30"/>
     </row>
-    <row r="87" spans="1:15" hidden="1">
+    <row r="87" spans="1:15">
       <c r="A87" s="31" t="s">
         <v>477</v>
       </c>
@@ -5442,7 +5463,7 @@
       <c r="N87" s="30"/>
       <c r="O87" s="30"/>
     </row>
-    <row r="88" spans="1:15" hidden="1">
+    <row r="88" spans="1:15">
       <c r="A88" s="31" t="s">
         <v>477</v>
       </c>
@@ -5473,7 +5494,7 @@
       <c r="N88" s="30"/>
       <c r="O88" s="30"/>
     </row>
-    <row r="89" spans="1:15" hidden="1">
+    <row r="89" spans="1:15">
       <c r="A89" s="31" t="s">
         <v>477</v>
       </c>
@@ -5502,7 +5523,7 @@
       <c r="N89" s="30"/>
       <c r="O89" s="30"/>
     </row>
-    <row r="90" spans="1:15" hidden="1">
+    <row r="90" spans="1:15">
       <c r="A90" s="31" t="s">
         <v>477</v>
       </c>
@@ -5531,7 +5552,7 @@
       <c r="N90" s="30"/>
       <c r="O90" s="30"/>
     </row>
-    <row r="91" spans="1:15" hidden="1">
+    <row r="91" spans="1:15">
       <c r="A91" s="31" t="s">
         <v>477</v>
       </c>
@@ -5560,7 +5581,7 @@
       <c r="N91" s="30"/>
       <c r="O91" s="30"/>
     </row>
-    <row r="92" spans="1:15" hidden="1">
+    <row r="92" spans="1:15">
       <c r="A92" s="31" t="s">
         <v>477</v>
       </c>
@@ -5589,7 +5610,7 @@
       <c r="N92" s="30"/>
       <c r="O92" s="30"/>
     </row>
-    <row r="93" spans="1:15" hidden="1">
+    <row r="93" spans="1:15">
       <c r="A93" s="31" t="s">
         <v>477</v>
       </c>
@@ -5618,7 +5639,7 @@
       <c r="N93" s="30"/>
       <c r="O93" s="30"/>
     </row>
-    <row r="94" spans="1:15" hidden="1">
+    <row r="94" spans="1:15">
       <c r="A94" s="31" t="s">
         <v>477</v>
       </c>
@@ -5647,7 +5668,7 @@
       <c r="N94" s="30"/>
       <c r="O94" s="30"/>
     </row>
-    <row r="95" spans="1:15" hidden="1">
+    <row r="95" spans="1:15">
       <c r="A95" s="31" t="s">
         <v>477</v>
       </c>
@@ -5678,7 +5699,7 @@
       <c r="N95" s="30"/>
       <c r="O95" s="30"/>
     </row>
-    <row r="96" spans="1:15" hidden="1">
+    <row r="96" spans="1:15">
       <c r="A96" s="31" t="s">
         <v>477</v>
       </c>
@@ -5709,7 +5730,7 @@
       <c r="N96" s="30"/>
       <c r="O96" s="30"/>
     </row>
-    <row r="97" spans="1:15" hidden="1">
+    <row r="97" spans="1:15">
       <c r="A97" s="31" t="s">
         <v>477</v>
       </c>
@@ -5740,7 +5761,7 @@
       <c r="N97" s="30"/>
       <c r="O97" s="30"/>
     </row>
-    <row r="98" spans="1:15" hidden="1">
+    <row r="98" spans="1:15">
       <c r="A98" s="31" t="s">
         <v>477</v>
       </c>
@@ -5771,7 +5792,7 @@
       <c r="N98" s="30"/>
       <c r="O98" s="30"/>
     </row>
-    <row r="99" spans="1:15" hidden="1">
+    <row r="99" spans="1:15">
       <c r="A99" s="31" t="s">
         <v>477</v>
       </c>
@@ -5802,7 +5823,7 @@
       <c r="N99" s="30"/>
       <c r="O99" s="30"/>
     </row>
-    <row r="100" spans="1:15" hidden="1">
+    <row r="100" spans="1:15">
       <c r="A100" s="31" t="s">
         <v>477</v>
       </c>
@@ -5833,7 +5854,7 @@
       <c r="N100" s="30"/>
       <c r="O100" s="30"/>
     </row>
-    <row r="101" spans="1:15" hidden="1">
+    <row r="101" spans="1:15">
       <c r="A101" s="31" t="s">
         <v>477</v>
       </c>
@@ -5864,7 +5885,7 @@
       <c r="N101" s="30"/>
       <c r="O101" s="30"/>
     </row>
-    <row r="102" spans="1:15" hidden="1">
+    <row r="102" spans="1:15">
       <c r="A102" s="31" t="s">
         <v>477</v>
       </c>
@@ -5895,7 +5916,7 @@
       <c r="N102" s="30"/>
       <c r="O102" s="30"/>
     </row>
-    <row r="103" spans="1:15" hidden="1">
+    <row r="103" spans="1:15">
       <c r="A103" s="31" t="s">
         <v>477</v>
       </c>
@@ -5926,7 +5947,7 @@
       <c r="N103" s="30"/>
       <c r="O103" s="30"/>
     </row>
-    <row r="104" spans="1:15" hidden="1">
+    <row r="104" spans="1:15">
       <c r="A104" s="31" t="s">
         <v>477</v>
       </c>
@@ -5957,7 +5978,7 @@
       <c r="N104" s="30"/>
       <c r="O104" s="30"/>
     </row>
-    <row r="105" spans="1:15" hidden="1">
+    <row r="105" spans="1:15">
       <c r="A105" s="31" t="s">
         <v>477</v>
       </c>
@@ -5988,7 +6009,7 @@
       <c r="N105" s="30"/>
       <c r="O105" s="30"/>
     </row>
-    <row r="106" spans="1:15" hidden="1">
+    <row r="106" spans="1:15">
       <c r="A106" s="31" t="s">
         <v>477</v>
       </c>
@@ -6019,7 +6040,7 @@
       <c r="N106" s="30"/>
       <c r="O106" s="30"/>
     </row>
-    <row r="107" spans="1:15" hidden="1">
+    <row r="107" spans="1:15">
       <c r="A107" s="31" t="s">
         <v>477</v>
       </c>
@@ -6050,7 +6071,7 @@
       <c r="N107" s="30"/>
       <c r="O107" s="30"/>
     </row>
-    <row r="108" spans="1:15" hidden="1">
+    <row r="108" spans="1:15">
       <c r="A108" s="31" t="s">
         <v>477</v>
       </c>
@@ -6081,7 +6102,7 @@
       <c r="N108" s="30"/>
       <c r="O108" s="30"/>
     </row>
-    <row r="109" spans="1:15" hidden="1">
+    <row r="109" spans="1:15">
       <c r="A109" s="31" t="s">
         <v>477</v>
       </c>
@@ -6110,7 +6131,7 @@
       <c r="N109" s="30"/>
       <c r="O109" s="30"/>
     </row>
-    <row r="110" spans="1:15" hidden="1">
+    <row r="110" spans="1:15">
       <c r="A110" s="31" t="s">
         <v>477</v>
       </c>
@@ -6139,7 +6160,7 @@
       <c r="N110" s="30"/>
       <c r="O110" s="30"/>
     </row>
-    <row r="111" spans="1:15" hidden="1">
+    <row r="111" spans="1:15">
       <c r="A111" s="31" t="s">
         <v>477</v>
       </c>
@@ -6168,7 +6189,7 @@
       <c r="N111" s="30"/>
       <c r="O111" s="30"/>
     </row>
-    <row r="112" spans="1:15" hidden="1">
+    <row r="112" spans="1:15">
       <c r="A112" s="31" t="s">
         <v>477</v>
       </c>
@@ -6197,7 +6218,7 @@
       <c r="N112" s="30"/>
       <c r="O112" s="30"/>
     </row>
-    <row r="113" spans="1:15" hidden="1">
+    <row r="113" spans="1:15">
       <c r="A113" s="31" t="s">
         <v>477</v>
       </c>
@@ -6226,7 +6247,7 @@
       <c r="N113" s="30"/>
       <c r="O113" s="30"/>
     </row>
-    <row r="114" spans="1:15" hidden="1">
+    <row r="114" spans="1:15">
       <c r="A114" s="31" t="s">
         <v>477</v>
       </c>
@@ -6255,7 +6276,7 @@
       <c r="N114" s="30"/>
       <c r="O114" s="30"/>
     </row>
-    <row r="115" spans="1:15" hidden="1">
+    <row r="115" spans="1:15">
       <c r="A115" s="31" t="s">
         <v>477</v>
       </c>
@@ -6284,7 +6305,7 @@
       <c r="N115" s="30"/>
       <c r="O115" s="30"/>
     </row>
-    <row r="116" spans="1:15" hidden="1">
+    <row r="116" spans="1:15">
       <c r="A116" s="31" t="s">
         <v>477</v>
       </c>
@@ -6313,7 +6334,7 @@
       <c r="N116" s="30"/>
       <c r="O116" s="30"/>
     </row>
-    <row r="117" spans="1:15" hidden="1">
+    <row r="117" spans="1:15">
       <c r="A117" s="31" t="s">
         <v>477</v>
       </c>
@@ -6342,7 +6363,7 @@
       <c r="N117" s="30"/>
       <c r="O117" s="30"/>
     </row>
-    <row r="118" spans="1:15" hidden="1">
+    <row r="118" spans="1:15">
       <c r="A118" s="31" t="s">
         <v>477</v>
       </c>
@@ -6371,7 +6392,7 @@
       <c r="N118" s="30"/>
       <c r="O118" s="30"/>
     </row>
-    <row r="119" spans="1:15" hidden="1">
+    <row r="119" spans="1:15">
       <c r="A119" s="31" t="s">
         <v>477</v>
       </c>
@@ -6400,7 +6421,7 @@
       <c r="N119" s="30"/>
       <c r="O119" s="30"/>
     </row>
-    <row r="120" spans="1:15" hidden="1">
+    <row r="120" spans="1:15">
       <c r="A120" s="31" t="s">
         <v>477</v>
       </c>
@@ -6429,7 +6450,7 @@
       <c r="N120" s="30"/>
       <c r="O120" s="30"/>
     </row>
-    <row r="121" spans="1:15" hidden="1">
+    <row r="121" spans="1:15">
       <c r="A121" s="31" t="s">
         <v>477</v>
       </c>
@@ -6462,7 +6483,7 @@
       <c r="N121" s="30"/>
       <c r="O121" s="30"/>
     </row>
-    <row r="122" spans="1:15" hidden="1">
+    <row r="122" spans="1:15">
       <c r="A122" s="31" t="s">
         <v>477</v>
       </c>
@@ -6493,7 +6514,7 @@
       <c r="N122" s="30"/>
       <c r="O122" s="30"/>
     </row>
-    <row r="123" spans="1:15" hidden="1">
+    <row r="123" spans="1:15">
       <c r="A123" s="31" t="s">
         <v>477</v>
       </c>
@@ -6524,7 +6545,7 @@
       <c r="N123" s="30"/>
       <c r="O123" s="30"/>
     </row>
-    <row r="124" spans="1:15" hidden="1">
+    <row r="124" spans="1:15">
       <c r="A124" s="31" t="s">
         <v>477</v>
       </c>
@@ -6555,7 +6576,7 @@
       <c r="N124" s="30"/>
       <c r="O124" s="30"/>
     </row>
-    <row r="125" spans="1:15" hidden="1">
+    <row r="125" spans="1:15">
       <c r="A125" s="31" t="s">
         <v>477</v>
       </c>
@@ -6586,7 +6607,7 @@
       <c r="N125" s="30"/>
       <c r="O125" s="30"/>
     </row>
-    <row r="126" spans="1:15" hidden="1">
+    <row r="126" spans="1:15">
       <c r="A126" s="31" t="s">
         <v>477</v>
       </c>
@@ -6617,7 +6638,7 @@
       <c r="N126" s="30"/>
       <c r="O126" s="30"/>
     </row>
-    <row r="127" spans="1:15" hidden="1">
+    <row r="127" spans="1:15">
       <c r="A127" s="31" t="s">
         <v>477</v>
       </c>
@@ -6648,7 +6669,7 @@
       <c r="N127" s="30"/>
       <c r="O127" s="30"/>
     </row>
-    <row r="128" spans="1:15" hidden="1">
+    <row r="128" spans="1:15">
       <c r="A128" s="31" t="s">
         <v>477</v>
       </c>
@@ -6679,7 +6700,7 @@
       <c r="N128" s="30"/>
       <c r="O128" s="30"/>
     </row>
-    <row r="129" spans="1:15" hidden="1">
+    <row r="129" spans="1:15">
       <c r="A129" s="31" t="s">
         <v>477</v>
       </c>
@@ -6710,7 +6731,7 @@
       <c r="N129" s="30"/>
       <c r="O129" s="30"/>
     </row>
-    <row r="130" spans="1:15" hidden="1">
+    <row r="130" spans="1:15">
       <c r="A130" s="31" t="s">
         <v>477</v>
       </c>
@@ -6741,7 +6762,7 @@
       <c r="N130" s="30"/>
       <c r="O130" s="30"/>
     </row>
-    <row r="131" spans="1:15" hidden="1">
+    <row r="131" spans="1:15" ht="28.8">
       <c r="A131" s="31" t="s">
         <v>477</v>
       </c>
@@ -6770,7 +6791,7 @@
       <c r="N131" s="30"/>
       <c r="O131" s="30"/>
     </row>
-    <row r="132" spans="1:15" hidden="1">
+    <row r="132" spans="1:15">
       <c r="A132" s="31" t="s">
         <v>477</v>
       </c>
@@ -6799,7 +6820,7 @@
       <c r="N132" s="30"/>
       <c r="O132" s="30"/>
     </row>
-    <row r="133" spans="1:15" hidden="1">
+    <row r="133" spans="1:15">
       <c r="A133" s="31" t="s">
         <v>477</v>
       </c>
@@ -6830,7 +6851,7 @@
       <c r="N133" s="30"/>
       <c r="O133" s="30"/>
     </row>
-    <row r="134" spans="1:15" hidden="1">
+    <row r="134" spans="1:15">
       <c r="A134" s="31" t="s">
         <v>477</v>
       </c>
@@ -6863,7 +6884,7 @@
       <c r="N134" s="30"/>
       <c r="O134" s="30"/>
     </row>
-    <row r="135" spans="1:15" hidden="1">
+    <row r="135" spans="1:15">
       <c r="A135" s="31" t="s">
         <v>477</v>
       </c>
@@ -6894,7 +6915,7 @@
       <c r="N135" s="30"/>
       <c r="O135" s="30"/>
     </row>
-    <row r="136" spans="1:15" hidden="1">
+    <row r="136" spans="1:15">
       <c r="A136" s="31" t="s">
         <v>477</v>
       </c>
@@ -6923,7 +6944,7 @@
       <c r="N136" s="30"/>
       <c r="O136" s="30"/>
     </row>
-    <row r="137" spans="1:15" hidden="1">
+    <row r="137" spans="1:15">
       <c r="A137" s="31" t="s">
         <v>477</v>
       </c>
@@ -6952,7 +6973,7 @@
       <c r="N137" s="30"/>
       <c r="O137" s="30"/>
     </row>
-    <row r="138" spans="1:15" hidden="1">
+    <row r="138" spans="1:15">
       <c r="A138" s="31" t="s">
         <v>477</v>
       </c>
@@ -6981,7 +7002,7 @@
       <c r="N138" s="30"/>
       <c r="O138" s="30"/>
     </row>
-    <row r="139" spans="1:15" hidden="1">
+    <row r="139" spans="1:15" ht="43.2">
       <c r="A139" s="31" t="s">
         <v>477</v>
       </c>
@@ -7010,7 +7031,7 @@
       <c r="N139" s="30"/>
       <c r="O139" s="30"/>
     </row>
-    <row r="140" spans="1:15" hidden="1">
+    <row r="140" spans="1:15">
       <c r="A140" s="31" t="s">
         <v>477</v>
       </c>
@@ -7039,7 +7060,7 @@
       <c r="N140" s="30"/>
       <c r="O140" s="30"/>
     </row>
-    <row r="141" spans="1:15" hidden="1">
+    <row r="141" spans="1:15" ht="43.2">
       <c r="A141" s="31" t="s">
         <v>477</v>
       </c>
@@ -7068,7 +7089,7 @@
       <c r="N141" s="30"/>
       <c r="O141" s="30"/>
     </row>
-    <row r="142" spans="1:15" hidden="1">
+    <row r="142" spans="1:15" ht="43.2">
       <c r="A142" s="31" t="s">
         <v>477</v>
       </c>
@@ -7097,7 +7118,7 @@
       <c r="N142" s="30"/>
       <c r="O142" s="30"/>
     </row>
-    <row r="143" spans="1:15" hidden="1">
+    <row r="143" spans="1:15">
       <c r="A143" s="31" t="s">
         <v>477</v>
       </c>
@@ -7126,7 +7147,7 @@
       <c r="N143" s="30"/>
       <c r="O143" s="30"/>
     </row>
-    <row r="144" spans="1:15" hidden="1">
+    <row r="144" spans="1:15" ht="43.2">
       <c r="A144" s="31" t="s">
         <v>477</v>
       </c>
@@ -7155,7 +7176,7 @@
       <c r="N144" s="30"/>
       <c r="O144" s="30"/>
     </row>
-    <row r="145" spans="1:15" hidden="1">
+    <row r="145" spans="1:15">
       <c r="A145" s="31" t="s">
         <v>477</v>
       </c>
@@ -7184,7 +7205,7 @@
       <c r="N145" s="30"/>
       <c r="O145" s="30"/>
     </row>
-    <row r="146" spans="1:15" hidden="1">
+    <row r="146" spans="1:15">
       <c r="A146" s="31" t="s">
         <v>477</v>
       </c>
@@ -7213,7 +7234,7 @@
       <c r="N146" s="30"/>
       <c r="O146" s="30"/>
     </row>
-    <row r="147" spans="1:15" hidden="1">
+    <row r="147" spans="1:15">
       <c r="A147" s="31" t="s">
         <v>477</v>
       </c>
@@ -7240,7 +7261,7 @@
       <c r="N147" s="30"/>
       <c r="O147" s="30"/>
     </row>
-    <row r="148" spans="1:15" hidden="1">
+    <row r="148" spans="1:15">
       <c r="A148" s="31" t="s">
         <v>477</v>
       </c>
@@ -7267,7 +7288,7 @@
       <c r="N148" s="30"/>
       <c r="O148" s="30"/>
     </row>
-    <row r="149" spans="1:15" hidden="1">
+    <row r="149" spans="1:15">
       <c r="A149" s="31" t="s">
         <v>477</v>
       </c>
@@ -7294,7 +7315,7 @@
       <c r="N149" s="30"/>
       <c r="O149" s="30"/>
     </row>
-    <row r="150" spans="1:15" hidden="1">
+    <row r="150" spans="1:15">
       <c r="A150" s="31" t="s">
         <v>477</v>
       </c>
@@ -7321,7 +7342,7 @@
       <c r="N150" s="30"/>
       <c r="O150" s="30"/>
     </row>
-    <row r="151" spans="1:15" hidden="1">
+    <row r="151" spans="1:15">
       <c r="A151" s="31" t="s">
         <v>477</v>
       </c>
@@ -7348,7 +7369,7 @@
       <c r="N151" s="30"/>
       <c r="O151" s="30"/>
     </row>
-    <row r="152" spans="1:15" hidden="1">
+    <row r="152" spans="1:15">
       <c r="A152" s="31" t="s">
         <v>477</v>
       </c>
@@ -7377,7 +7398,7 @@
       <c r="N152" s="30"/>
       <c r="O152" s="30"/>
     </row>
-    <row r="153" spans="1:15" hidden="1">
+    <row r="153" spans="1:15">
       <c r="A153" s="31" t="s">
         <v>477</v>
       </c>
@@ -7406,7 +7427,7 @@
       <c r="N153" s="30"/>
       <c r="O153" s="30"/>
     </row>
-    <row r="154" spans="1:15" hidden="1">
+    <row r="154" spans="1:15">
       <c r="A154" s="31" t="s">
         <v>477</v>
       </c>
@@ -7435,7 +7456,7 @@
       <c r="N154" s="30"/>
       <c r="O154" s="30"/>
     </row>
-    <row r="155" spans="1:15" hidden="1">
+    <row r="155" spans="1:15">
       <c r="A155" s="31" t="s">
         <v>477</v>
       </c>
@@ -7462,7 +7483,7 @@
       <c r="N155" s="30"/>
       <c r="O155" s="30"/>
     </row>
-    <row r="156" spans="1:15" hidden="1">
+    <row r="156" spans="1:15">
       <c r="A156" s="31" t="s">
         <v>477</v>
       </c>
@@ -7489,7 +7510,7 @@
       <c r="N156" s="30"/>
       <c r="O156" s="30"/>
     </row>
-    <row r="157" spans="1:15" hidden="1">
+    <row r="157" spans="1:15">
       <c r="A157" s="31" t="s">
         <v>477</v>
       </c>
@@ -7516,7 +7537,7 @@
       <c r="N157" s="30"/>
       <c r="O157" s="30"/>
     </row>
-    <row r="158" spans="1:15" hidden="1">
+    <row r="158" spans="1:15">
       <c r="A158" s="31" t="s">
         <v>477</v>
       </c>
@@ -7543,7 +7564,7 @@
       <c r="N158" s="30"/>
       <c r="O158" s="30"/>
     </row>
-    <row r="159" spans="1:15" hidden="1">
+    <row r="159" spans="1:15">
       <c r="A159" s="31" t="s">
         <v>477</v>
       </c>
@@ -7570,7 +7591,7 @@
       <c r="N159" s="30"/>
       <c r="O159" s="30"/>
     </row>
-    <row r="160" spans="1:15" hidden="1">
+    <row r="160" spans="1:15" ht="28.8">
       <c r="A160" s="31" t="s">
         <v>477</v>
       </c>
@@ -7597,7 +7618,7 @@
       <c r="N160" s="30"/>
       <c r="O160" s="30"/>
     </row>
-    <row r="161" spans="1:15" hidden="1">
+    <row r="161" spans="1:15">
       <c r="A161" s="31" t="s">
         <v>477</v>
       </c>
@@ -7624,7 +7645,7 @@
       <c r="N161" s="30"/>
       <c r="O161" s="30"/>
     </row>
-    <row r="162" spans="1:15" ht="13.5" hidden="1" customHeight="1">
+    <row r="162" spans="1:15" ht="13.5" customHeight="1">
       <c r="A162" s="31" t="s">
         <v>477</v>
       </c>
@@ -7653,7 +7674,7 @@
       <c r="N162" s="30"/>
       <c r="O162" s="30"/>
     </row>
-    <row r="163" spans="1:15" ht="13.5" hidden="1" customHeight="1">
+    <row r="163" spans="1:15" ht="13.5" customHeight="1">
       <c r="A163" s="31" t="s">
         <v>477</v>
       </c>
@@ -7680,7 +7701,7 @@
       <c r="N163" s="30"/>
       <c r="O163" s="30"/>
     </row>
-    <row r="164" spans="1:15" ht="13.5" hidden="1" customHeight="1">
+    <row r="164" spans="1:15" ht="13.5" customHeight="1">
       <c r="A164" s="31" t="s">
         <v>477</v>
       </c>
@@ -7707,7 +7728,7 @@
       <c r="N164" s="30"/>
       <c r="O164" s="30"/>
     </row>
-    <row r="165" spans="1:15" hidden="1">
+    <row r="165" spans="1:15" ht="28.8">
       <c r="A165" s="31" t="s">
         <v>477</v>
       </c>
@@ -7736,7 +7757,7 @@
       <c r="N165" s="30"/>
       <c r="O165" s="30"/>
     </row>
-    <row r="166" spans="1:15" hidden="1">
+    <row r="166" spans="1:15">
       <c r="A166" s="31" t="s">
         <v>477</v>
       </c>
@@ -7763,7 +7784,7 @@
       <c r="N166" s="30"/>
       <c r="O166" s="30"/>
     </row>
-    <row r="167" spans="1:15" hidden="1">
+    <row r="167" spans="1:15">
       <c r="A167" s="31" t="s">
         <v>477</v>
       </c>
@@ -7790,7 +7811,7 @@
       <c r="N167" s="30"/>
       <c r="O167" s="30"/>
     </row>
-    <row r="168" spans="1:15" hidden="1">
+    <row r="168" spans="1:15">
       <c r="A168" s="31" t="s">
         <v>477</v>
       </c>
@@ -7817,7 +7838,7 @@
       <c r="N168" s="30"/>
       <c r="O168" s="30"/>
     </row>
-    <row r="169" spans="1:15" hidden="1">
+    <row r="169" spans="1:15">
       <c r="A169" s="31" t="s">
         <v>477</v>
       </c>
@@ -7844,7 +7865,7 @@
       <c r="N169" s="30"/>
       <c r="O169" s="30"/>
     </row>
-    <row r="170" spans="1:15" hidden="1">
+    <row r="170" spans="1:15">
       <c r="A170" s="31" t="s">
         <v>477</v>
       </c>
@@ -7871,7 +7892,7 @@
       <c r="N170" s="30"/>
       <c r="O170" s="30"/>
     </row>
-    <row r="171" spans="1:15" hidden="1">
+    <row r="171" spans="1:15">
       <c r="A171" s="31" t="s">
         <v>477</v>
       </c>
@@ -7898,7 +7919,7 @@
       <c r="N171" s="30"/>
       <c r="O171" s="30"/>
     </row>
-    <row r="172" spans="1:15" hidden="1">
+    <row r="172" spans="1:15">
       <c r="A172" s="31" t="s">
         <v>477</v>
       </c>
@@ -7925,7 +7946,7 @@
       <c r="N172" s="30"/>
       <c r="O172" s="30"/>
     </row>
-    <row r="173" spans="1:15" hidden="1">
+    <row r="173" spans="1:15">
       <c r="A173" s="31" t="s">
         <v>477</v>
       </c>
@@ -7954,7 +7975,7 @@
       <c r="N173" s="30"/>
       <c r="O173" s="30"/>
     </row>
-    <row r="174" spans="1:15" hidden="1">
+    <row r="174" spans="1:15">
       <c r="A174" s="31" t="s">
         <v>477</v>
       </c>
@@ -7987,7 +8008,7 @@
       <c r="N174" s="30"/>
       <c r="O174" s="30"/>
     </row>
-    <row r="175" spans="1:15" hidden="1">
+    <row r="175" spans="1:15">
       <c r="A175" s="31" t="s">
         <v>477</v>
       </c>
@@ -8016,7 +8037,7 @@
       <c r="N175" s="30"/>
       <c r="O175" s="30"/>
     </row>
-    <row r="176" spans="1:15" hidden="1">
+    <row r="176" spans="1:15">
       <c r="A176" s="31" t="s">
         <v>477</v>
       </c>
@@ -8045,7 +8066,7 @@
       <c r="N176" s="30"/>
       <c r="O176" s="30"/>
     </row>
-    <row r="177" spans="1:15" hidden="1">
+    <row r="177" spans="1:15">
       <c r="A177" s="31" t="s">
         <v>477</v>
       </c>
@@ -8076,7 +8097,7 @@
       <c r="N177" s="30"/>
       <c r="O177" s="30"/>
     </row>
-    <row r="178" spans="1:15" hidden="1">
+    <row r="178" spans="1:15">
       <c r="A178" s="31" t="s">
         <v>477</v>
       </c>
@@ -8107,7 +8128,7 @@
       <c r="N178" s="30"/>
       <c r="O178" s="30"/>
     </row>
-    <row r="179" spans="1:15" hidden="1">
+    <row r="179" spans="1:15">
       <c r="A179" s="31" t="s">
         <v>477</v>
       </c>
@@ -8138,7 +8159,7 @@
       <c r="N179" s="30"/>
       <c r="O179" s="30"/>
     </row>
-    <row r="180" spans="1:15" hidden="1">
+    <row r="180" spans="1:15">
       <c r="A180" s="31" t="s">
         <v>477</v>
       </c>
@@ -8169,7 +8190,7 @@
       <c r="N180" s="30"/>
       <c r="O180" s="30"/>
     </row>
-    <row r="181" spans="1:15" hidden="1">
+    <row r="181" spans="1:15">
       <c r="A181" s="31" t="s">
         <v>477</v>
       </c>
@@ -8200,7 +8221,7 @@
       <c r="N181" s="30"/>
       <c r="O181" s="30"/>
     </row>
-    <row r="182" spans="1:15" hidden="1">
+    <row r="182" spans="1:15">
       <c r="A182" s="31" t="s">
         <v>477</v>
       </c>
@@ -8231,7 +8252,7 @@
       <c r="N182" s="30"/>
       <c r="O182" s="30"/>
     </row>
-    <row r="183" spans="1:15" hidden="1">
+    <row r="183" spans="1:15">
       <c r="A183" s="31" t="s">
         <v>477</v>
       </c>
@@ -8262,7 +8283,7 @@
       <c r="N183" s="30"/>
       <c r="O183" s="30"/>
     </row>
-    <row r="184" spans="1:15" hidden="1">
+    <row r="184" spans="1:15">
       <c r="A184" s="31" t="s">
         <v>477</v>
       </c>
@@ -8293,7 +8314,7 @@
       <c r="N184" s="30"/>
       <c r="O184" s="30"/>
     </row>
-    <row r="185" spans="1:15" hidden="1">
+    <row r="185" spans="1:15">
       <c r="A185" s="31" t="s">
         <v>477</v>
       </c>
@@ -8324,7 +8345,7 @@
       <c r="N185" s="30"/>
       <c r="O185" s="30"/>
     </row>
-    <row r="186" spans="1:15" hidden="1">
+    <row r="186" spans="1:15">
       <c r="A186" s="31" t="s">
         <v>477</v>
       </c>
@@ -8355,7 +8376,7 @@
       <c r="N186" s="30"/>
       <c r="O186" s="30"/>
     </row>
-    <row r="187" spans="1:15" hidden="1">
+    <row r="187" spans="1:15">
       <c r="A187" s="31" t="s">
         <v>477</v>
       </c>
@@ -8386,7 +8407,7 @@
       <c r="N187" s="30"/>
       <c r="O187" s="30"/>
     </row>
-    <row r="188" spans="1:15" hidden="1">
+    <row r="188" spans="1:15">
       <c r="A188" s="31" t="s">
         <v>477</v>
       </c>
@@ -8417,7 +8438,7 @@
       <c r="N188" s="30"/>
       <c r="O188" s="30"/>
     </row>
-    <row r="189" spans="1:15" hidden="1">
+    <row r="189" spans="1:15">
       <c r="A189" s="31" t="s">
         <v>477</v>
       </c>
@@ -8448,7 +8469,7 @@
       <c r="N189" s="30"/>
       <c r="O189" s="30"/>
     </row>
-    <row r="190" spans="1:15" hidden="1">
+    <row r="190" spans="1:15">
       <c r="A190" s="31" t="s">
         <v>477</v>
       </c>
@@ -8479,7 +8500,7 @@
       <c r="N190" s="30"/>
       <c r="O190" s="30"/>
     </row>
-    <row r="191" spans="1:15" hidden="1">
+    <row r="191" spans="1:15">
       <c r="A191" s="31" t="s">
         <v>477</v>
       </c>
@@ -8510,7 +8531,7 @@
       <c r="N191" s="30"/>
       <c r="O191" s="30"/>
     </row>
-    <row r="192" spans="1:15" hidden="1">
+    <row r="192" spans="1:15">
       <c r="A192" s="31" t="s">
         <v>477</v>
       </c>
@@ -8541,7 +8562,7 @@
       <c r="N192" s="30"/>
       <c r="O192" s="30"/>
     </row>
-    <row r="193" spans="1:15" hidden="1">
+    <row r="193" spans="1:15">
       <c r="A193" s="31" t="s">
         <v>477</v>
       </c>
@@ -8572,7 +8593,7 @@
       <c r="N193" s="30"/>
       <c r="O193" s="30"/>
     </row>
-    <row r="194" spans="1:15" hidden="1">
+    <row r="194" spans="1:15">
       <c r="A194" s="31" t="s">
         <v>477</v>
       </c>
@@ -8603,7 +8624,7 @@
       <c r="N194" s="30"/>
       <c r="O194" s="30"/>
     </row>
-    <row r="195" spans="1:15" hidden="1">
+    <row r="195" spans="1:15">
       <c r="A195" s="31" t="s">
         <v>477</v>
       </c>
@@ -8634,7 +8655,7 @@
       <c r="N195" s="30"/>
       <c r="O195" s="30"/>
     </row>
-    <row r="196" spans="1:15" hidden="1">
+    <row r="196" spans="1:15">
       <c r="A196" s="31" t="s">
         <v>477</v>
       </c>
@@ -8665,7 +8686,7 @@
       <c r="N196" s="30"/>
       <c r="O196" s="30"/>
     </row>
-    <row r="197" spans="1:15" hidden="1">
+    <row r="197" spans="1:15">
       <c r="A197" s="31" t="s">
         <v>477</v>
       </c>
@@ -8696,7 +8717,7 @@
       <c r="N197" s="30"/>
       <c r="O197" s="30"/>
     </row>
-    <row r="198" spans="1:15" hidden="1">
+    <row r="198" spans="1:15">
       <c r="A198" s="31" t="s">
         <v>477</v>
       </c>
@@ -8727,7 +8748,7 @@
       <c r="N198" s="30"/>
       <c r="O198" s="30"/>
     </row>
-    <row r="199" spans="1:15" hidden="1">
+    <row r="199" spans="1:15">
       <c r="A199" s="31" t="s">
         <v>477</v>
       </c>
@@ -8758,7 +8779,7 @@
       <c r="N199" s="30"/>
       <c r="O199" s="30"/>
     </row>
-    <row r="200" spans="1:15" hidden="1">
+    <row r="200" spans="1:15">
       <c r="A200" s="31" t="s">
         <v>477</v>
       </c>
@@ -8789,7 +8810,7 @@
       <c r="N200" s="30"/>
       <c r="O200" s="30"/>
     </row>
-    <row r="201" spans="1:15" hidden="1">
+    <row r="201" spans="1:15">
       <c r="A201" s="31" t="s">
         <v>477</v>
       </c>
@@ -8820,7 +8841,7 @@
       <c r="N201" s="30"/>
       <c r="O201" s="30"/>
     </row>
-    <row r="202" spans="1:15" hidden="1">
+    <row r="202" spans="1:15">
       <c r="A202" s="31" t="s">
         <v>477</v>
       </c>
@@ -8851,7 +8872,7 @@
       <c r="N202" s="30"/>
       <c r="O202" s="30"/>
     </row>
-    <row r="203" spans="1:15" hidden="1">
+    <row r="203" spans="1:15">
       <c r="A203" s="31" t="s">
         <v>477</v>
       </c>
@@ -8882,7 +8903,7 @@
       <c r="N203" s="30"/>
       <c r="O203" s="30"/>
     </row>
-    <row r="204" spans="1:15" hidden="1">
+    <row r="204" spans="1:15">
       <c r="A204" s="31" t="s">
         <v>477</v>
       </c>
@@ -8913,7 +8934,7 @@
       <c r="N204" s="30"/>
       <c r="O204" s="30"/>
     </row>
-    <row r="205" spans="1:15" hidden="1">
+    <row r="205" spans="1:15">
       <c r="A205" s="31" t="s">
         <v>477</v>
       </c>
@@ -8944,7 +8965,7 @@
       <c r="N205" s="30"/>
       <c r="O205" s="30"/>
     </row>
-    <row r="206" spans="1:15" hidden="1">
+    <row r="206" spans="1:15">
       <c r="A206" s="31" t="s">
         <v>477</v>
       </c>
@@ -8975,7 +8996,7 @@
       <c r="N206" s="30"/>
       <c r="O206" s="30"/>
     </row>
-    <row r="207" spans="1:15" hidden="1">
+    <row r="207" spans="1:15">
       <c r="A207" s="31" t="s">
         <v>477</v>
       </c>
@@ -9006,7 +9027,7 @@
       <c r="N207" s="30"/>
       <c r="O207" s="30"/>
     </row>
-    <row r="208" spans="1:15" hidden="1">
+    <row r="208" spans="1:15">
       <c r="A208" s="31" t="s">
         <v>477</v>
       </c>
@@ -9037,7 +9058,7 @@
       <c r="N208" s="30"/>
       <c r="O208" s="30"/>
     </row>
-    <row r="209" spans="1:15" hidden="1">
+    <row r="209" spans="1:15">
       <c r="A209" s="31" t="s">
         <v>477</v>
       </c>
@@ -9068,7 +9089,7 @@
       <c r="N209" s="30"/>
       <c r="O209" s="30"/>
     </row>
-    <row r="210" spans="1:15" hidden="1">
+    <row r="210" spans="1:15">
       <c r="A210" s="31" t="s">
         <v>477</v>
       </c>
@@ -9099,7 +9120,7 @@
       <c r="N210" s="30"/>
       <c r="O210" s="30"/>
     </row>
-    <row r="211" spans="1:15" hidden="1">
+    <row r="211" spans="1:15">
       <c r="A211" s="31" t="s">
         <v>477</v>
       </c>
@@ -9130,7 +9151,7 @@
       <c r="N211" s="30"/>
       <c r="O211" s="30"/>
     </row>
-    <row r="212" spans="1:15" hidden="1">
+    <row r="212" spans="1:15">
       <c r="A212" s="31" t="s">
         <v>477</v>
       </c>
@@ -9161,7 +9182,7 @@
       <c r="N212" s="30"/>
       <c r="O212" s="30"/>
     </row>
-    <row r="213" spans="1:15" hidden="1">
+    <row r="213" spans="1:15">
       <c r="A213" s="31" t="s">
         <v>477</v>
       </c>
@@ -9192,7 +9213,7 @@
       <c r="N213" s="30"/>
       <c r="O213" s="30"/>
     </row>
-    <row r="214" spans="1:15" hidden="1">
+    <row r="214" spans="1:15">
       <c r="A214" s="31" t="s">
         <v>477</v>
       </c>
@@ -9223,7 +9244,7 @@
       <c r="N214" s="30"/>
       <c r="O214" s="30"/>
     </row>
-    <row r="215" spans="1:15" hidden="1">
+    <row r="215" spans="1:15">
       <c r="A215" s="31" t="s">
         <v>477</v>
       </c>
@@ -9254,7 +9275,7 @@
       <c r="N215" s="30"/>
       <c r="O215" s="30"/>
     </row>
-    <row r="216" spans="1:15" hidden="1">
+    <row r="216" spans="1:15">
       <c r="A216" s="31" t="s">
         <v>477</v>
       </c>
@@ -9285,7 +9306,7 @@
       <c r="N216" s="30"/>
       <c r="O216" s="30"/>
     </row>
-    <row r="217" spans="1:15" hidden="1">
+    <row r="217" spans="1:15">
       <c r="A217" s="31" t="s">
         <v>477</v>
       </c>
@@ -9316,7 +9337,7 @@
       <c r="N217" s="30"/>
       <c r="O217" s="30"/>
     </row>
-    <row r="218" spans="1:15" hidden="1">
+    <row r="218" spans="1:15">
       <c r="A218" s="31" t="s">
         <v>477</v>
       </c>
@@ -9347,7 +9368,7 @@
       <c r="N218" s="30"/>
       <c r="O218" s="30"/>
     </row>
-    <row r="219" spans="1:15" hidden="1">
+    <row r="219" spans="1:15">
       <c r="A219" s="31" t="s">
         <v>477</v>
       </c>
@@ -9378,7 +9399,7 @@
       <c r="N219" s="30"/>
       <c r="O219" s="30"/>
     </row>
-    <row r="220" spans="1:15" hidden="1">
+    <row r="220" spans="1:15">
       <c r="A220" s="31" t="s">
         <v>477</v>
       </c>
@@ -9409,7 +9430,7 @@
       <c r="N220" s="30"/>
       <c r="O220" s="30"/>
     </row>
-    <row r="221" spans="1:15" hidden="1">
+    <row r="221" spans="1:15">
       <c r="A221" s="31" t="s">
         <v>477</v>
       </c>
@@ -9440,7 +9461,7 @@
       <c r="N221" s="30"/>
       <c r="O221" s="30"/>
     </row>
-    <row r="222" spans="1:15" hidden="1">
+    <row r="222" spans="1:15">
       <c r="A222" s="31" t="s">
         <v>477</v>
       </c>
@@ -9471,7 +9492,7 @@
       <c r="N222" s="30"/>
       <c r="O222" s="30"/>
     </row>
-    <row r="223" spans="1:15" hidden="1">
+    <row r="223" spans="1:15">
       <c r="A223" s="31" t="s">
         <v>477</v>
       </c>
@@ -9502,7 +9523,7 @@
       <c r="N223" s="30"/>
       <c r="O223" s="30"/>
     </row>
-    <row r="224" spans="1:15" hidden="1">
+    <row r="224" spans="1:15">
       <c r="A224" s="31" t="s">
         <v>477</v>
       </c>
@@ -9533,7 +9554,7 @@
       <c r="N224" s="30"/>
       <c r="O224" s="30"/>
     </row>
-    <row r="225" spans="1:15" hidden="1">
+    <row r="225" spans="1:15">
       <c r="A225" s="31" t="s">
         <v>477</v>
       </c>
@@ -9564,7 +9585,7 @@
       <c r="N225" s="30"/>
       <c r="O225" s="30"/>
     </row>
-    <row r="226" spans="1:15" hidden="1">
+    <row r="226" spans="1:15">
       <c r="A226" s="31" t="s">
         <v>477</v>
       </c>
@@ -9595,7 +9616,7 @@
       <c r="N226" s="30"/>
       <c r="O226" s="30"/>
     </row>
-    <row r="227" spans="1:15" hidden="1">
+    <row r="227" spans="1:15">
       <c r="A227" s="31" t="s">
         <v>477</v>
       </c>
@@ -9626,7 +9647,7 @@
       <c r="N227" s="30"/>
       <c r="O227" s="30"/>
     </row>
-    <row r="228" spans="1:15" hidden="1">
+    <row r="228" spans="1:15">
       <c r="A228" s="31" t="s">
         <v>477</v>
       </c>
@@ -9657,7 +9678,7 @@
       <c r="N228" s="30"/>
       <c r="O228" s="30"/>
     </row>
-    <row r="229" spans="1:15" hidden="1">
+    <row r="229" spans="1:15">
       <c r="A229" s="31" t="s">
         <v>477</v>
       </c>
@@ -9688,7 +9709,7 @@
       <c r="N229" s="30"/>
       <c r="O229" s="30"/>
     </row>
-    <row r="230" spans="1:15" hidden="1">
+    <row r="230" spans="1:15">
       <c r="A230" s="31" t="s">
         <v>477</v>
       </c>
@@ -9719,7 +9740,7 @@
       <c r="N230" s="30"/>
       <c r="O230" s="30"/>
     </row>
-    <row r="231" spans="1:15" hidden="1">
+    <row r="231" spans="1:15">
       <c r="A231" s="31" t="s">
         <v>477</v>
       </c>
@@ -9750,7 +9771,7 @@
       <c r="N231" s="30"/>
       <c r="O231" s="30"/>
     </row>
-    <row r="232" spans="1:15" hidden="1">
+    <row r="232" spans="1:15">
       <c r="A232" s="31" t="s">
         <v>477</v>
       </c>
@@ -9781,7 +9802,7 @@
       <c r="N232" s="30"/>
       <c r="O232" s="30"/>
     </row>
-    <row r="233" spans="1:15" hidden="1">
+    <row r="233" spans="1:15">
       <c r="A233" s="31" t="s">
         <v>477</v>
       </c>
@@ -9812,7 +9833,7 @@
       <c r="N233" s="30"/>
       <c r="O233" s="30"/>
     </row>
-    <row r="234" spans="1:15" hidden="1">
+    <row r="234" spans="1:15">
       <c r="A234" s="31" t="s">
         <v>477</v>
       </c>
@@ -9843,7 +9864,7 @@
       <c r="N234" s="30"/>
       <c r="O234" s="30"/>
     </row>
-    <row r="235" spans="1:15" hidden="1">
+    <row r="235" spans="1:15">
       <c r="A235" s="31" t="s">
         <v>477</v>
       </c>
@@ -9874,7 +9895,7 @@
       <c r="N235" s="30"/>
       <c r="O235" s="30"/>
     </row>
-    <row r="236" spans="1:15" hidden="1">
+    <row r="236" spans="1:15">
       <c r="A236" s="31" t="s">
         <v>477</v>
       </c>
@@ -9905,7 +9926,7 @@
       <c r="N236" s="30"/>
       <c r="O236" s="30"/>
     </row>
-    <row r="237" spans="1:15" hidden="1">
+    <row r="237" spans="1:15">
       <c r="A237" s="31" t="s">
         <v>477</v>
       </c>
@@ -9936,7 +9957,7 @@
       <c r="N237" s="30"/>
       <c r="O237" s="30"/>
     </row>
-    <row r="238" spans="1:15" hidden="1">
+    <row r="238" spans="1:15">
       <c r="A238" s="31" t="s">
         <v>477</v>
       </c>
@@ -9967,7 +9988,7 @@
       <c r="N238" s="30"/>
       <c r="O238" s="30"/>
     </row>
-    <row r="239" spans="1:15" hidden="1">
+    <row r="239" spans="1:15">
       <c r="A239" s="31" t="s">
         <v>477</v>
       </c>
@@ -9998,7 +10019,7 @@
       <c r="N239" s="30"/>
       <c r="O239" s="30"/>
     </row>
-    <row r="240" spans="1:15" hidden="1">
+    <row r="240" spans="1:15" ht="28.8">
       <c r="A240" s="31" t="s">
         <v>477</v>
       </c>
@@ -10029,7 +10050,7 @@
       <c r="N240" s="30"/>
       <c r="O240" s="30"/>
     </row>
-    <row r="241" spans="1:15" hidden="1">
+    <row r="241" spans="1:15" ht="28.8">
       <c r="A241" s="31" t="s">
         <v>477</v>
       </c>
@@ -10060,7 +10081,7 @@
       <c r="N241" s="30"/>
       <c r="O241" s="30"/>
     </row>
-    <row r="242" spans="1:15" hidden="1">
+    <row r="242" spans="1:15" ht="28.8">
       <c r="A242" s="31" t="s">
         <v>477</v>
       </c>
@@ -10091,7 +10112,7 @@
       <c r="N242" s="30"/>
       <c r="O242" s="30"/>
     </row>
-    <row r="243" spans="1:15" hidden="1">
+    <row r="243" spans="1:15">
       <c r="A243" s="31" t="s">
         <v>477</v>
       </c>
@@ -10122,7 +10143,7 @@
       <c r="N243" s="30"/>
       <c r="O243" s="30"/>
     </row>
-    <row r="244" spans="1:15" hidden="1">
+    <row r="244" spans="1:15" ht="28.8">
       <c r="A244" s="31" t="s">
         <v>477</v>
       </c>
@@ -10153,7 +10174,7 @@
       <c r="N244" s="30"/>
       <c r="O244" s="30"/>
     </row>
-    <row r="245" spans="1:15" hidden="1">
+    <row r="245" spans="1:15">
       <c r="A245" s="31" t="s">
         <v>477</v>
       </c>
@@ -10184,7 +10205,7 @@
       <c r="N245" s="30"/>
       <c r="O245" s="30"/>
     </row>
-    <row r="246" spans="1:15" hidden="1">
+    <row r="246" spans="1:15">
       <c r="A246" s="31" t="s">
         <v>477</v>
       </c>
@@ -10215,7 +10236,7 @@
       <c r="N246" s="30"/>
       <c r="O246" s="30"/>
     </row>
-    <row r="247" spans="1:15" hidden="1">
+    <row r="247" spans="1:15">
       <c r="A247" s="31" t="s">
         <v>477</v>
       </c>
@@ -10246,7 +10267,7 @@
       <c r="N247" s="30"/>
       <c r="O247" s="30"/>
     </row>
-    <row r="248" spans="1:15" hidden="1">
+    <row r="248" spans="1:15">
       <c r="A248" s="31" t="s">
         <v>477</v>
       </c>
@@ -10277,7 +10298,7 @@
       <c r="N248" s="30"/>
       <c r="O248" s="30"/>
     </row>
-    <row r="249" spans="1:15" hidden="1">
+    <row r="249" spans="1:15">
       <c r="A249" s="31" t="s">
         <v>477</v>
       </c>
@@ -10308,7 +10329,7 @@
       <c r="N249" s="30"/>
       <c r="O249" s="30"/>
     </row>
-    <row r="250" spans="1:15" hidden="1">
+    <row r="250" spans="1:15">
       <c r="A250" s="31" t="s">
         <v>477</v>
       </c>
@@ -10339,7 +10360,7 @@
       <c r="N250" s="30"/>
       <c r="O250" s="30"/>
     </row>
-    <row r="251" spans="1:15" hidden="1">
+    <row r="251" spans="1:15" ht="28.8">
       <c r="A251" s="31" t="s">
         <v>477</v>
       </c>
@@ -10372,7 +10393,7 @@
       <c r="N251" s="30"/>
       <c r="O251" s="30"/>
     </row>
-    <row r="252" spans="1:15" hidden="1">
+    <row r="252" spans="1:15">
       <c r="A252" s="31" t="s">
         <v>477</v>
       </c>
@@ -10405,7 +10426,7 @@
       <c r="N252" s="30"/>
       <c r="O252" s="30"/>
     </row>
-    <row r="253" spans="1:15" hidden="1">
+    <row r="253" spans="1:15">
       <c r="A253" s="31" t="s">
         <v>477</v>
       </c>
@@ -10438,7 +10459,7 @@
       <c r="N253" s="30"/>
       <c r="O253" s="30"/>
     </row>
-    <row r="254" spans="1:15" hidden="1">
+    <row r="254" spans="1:15">
       <c r="A254" s="31" t="s">
         <v>477</v>
       </c>
@@ -10471,7 +10492,7 @@
       <c r="N254" s="30"/>
       <c r="O254" s="30"/>
     </row>
-    <row r="255" spans="1:15" hidden="1">
+    <row r="255" spans="1:15">
       <c r="A255" s="31" t="s">
         <v>477</v>
       </c>
@@ -10504,7 +10525,7 @@
       <c r="N255" s="30"/>
       <c r="O255" s="30"/>
     </row>
-    <row r="256" spans="1:15" hidden="1">
+    <row r="256" spans="1:15">
       <c r="A256" s="31" t="s">
         <v>477</v>
       </c>
@@ -10537,7 +10558,7 @@
       <c r="N256" s="30"/>
       <c r="O256" s="30"/>
     </row>
-    <row r="257" spans="1:15" hidden="1">
+    <row r="257" spans="1:15">
       <c r="A257" s="31" t="s">
         <v>477</v>
       </c>
@@ -10570,7 +10591,7 @@
       <c r="N257" s="30"/>
       <c r="O257" s="30"/>
     </row>
-    <row r="258" spans="1:15" ht="15" hidden="1" customHeight="1">
+    <row r="258" spans="1:15" ht="15" customHeight="1">
       <c r="A258" s="31" t="s">
         <v>477</v>
       </c>
@@ -10603,7 +10624,7 @@
       <c r="N258" s="30"/>
       <c r="O258" s="30"/>
     </row>
-    <row r="259" spans="1:15" ht="16.5" hidden="1" customHeight="1">
+    <row r="259" spans="1:15" ht="16.5" customHeight="1">
       <c r="A259" s="31" t="s">
         <v>477</v>
       </c>
@@ -10640,7 +10661,7 @@
   <autoFilter ref="A1:O259" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Cuidado corporal (1)"/>
+        <filter val="Hogar y bienestar (3)"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -10711,7 +10732,7 @@
         <v>Limpiadores faciales-10</v>
       </c>
       <c r="C2" t="str" cm="1">
-        <f t="array" ref="C2:C19">_xlfn.UNIQUE(Avance!C2:C259,FALSE,FALSE)</f>
+        <f t="array" ref="C2:C20">_xlfn.UNIQUE(Avance!C2:C259,FALSE,FALSE)</f>
         <v>Agua Micelar</v>
       </c>
       <c r="D2" t="str" cm="1">
@@ -10857,7 +10878,7 @@
         <v>Serum-14</v>
       </c>
       <c r="C6" t="str">
-        <v>Golden Collection</v>
+        <v>Basic Essences Collection (11)</v>
       </c>
       <c r="D6" t="str">
         <v>Piel Sensible</v>
@@ -10884,7 +10905,7 @@
         <v>Productos para los ojos-15</v>
       </c>
       <c r="C7" t="str">
-        <v>Beauty Words Collection</v>
+        <v>Golden Collection</v>
       </c>
       <c r="D7" t="str">
         <v>Productos para pestañas</v>
@@ -10910,7 +10931,7 @@
         <v>Hidratante de labios-16</v>
       </c>
       <c r="C8" t="str">
-        <v>Angel Numbers Collection</v>
+        <v>Beauty Words Collection</v>
       </c>
       <c r="D8" t="str">
         <v>Productos para labios</v>
@@ -10934,7 +10955,7 @@
         <v>Pasta dental-1</v>
       </c>
       <c r="C9" t="str">
-        <v>Manifest | Good &amp; Positive</v>
+        <v>Angel Numbers Collection</v>
       </c>
       <c r="D9" t="str">
         <v>Cuidado personal</v>
@@ -10960,7 +10981,7 @@
         <v>Crema de Manos-3</v>
       </c>
       <c r="C10" t="str">
-        <v>7 Chackras</v>
+        <v>Manifest | Good &amp; Positive</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -10981,7 +11002,7 @@
         <v>Crema de Cuerpo-4</v>
       </c>
       <c r="C11" t="str">
-        <v>Mood Candles</v>
+        <v>7 Chackras</v>
       </c>
       <c r="D11" t="str">
         <v>Cabello graso</v>
@@ -11001,7 +11022,7 @@
         <v>Desodorante-5</v>
       </c>
       <c r="C12" t="str">
-        <v>Difusores de varillas</v>
+        <v>Mood Candles</v>
       </c>
       <c r="D12" t="str">
         <v>Anti-celulitis</v>
@@ -11019,7 +11040,7 @@
         <v>Shampoo-6</v>
       </c>
       <c r="C13" t="str">
-        <v>Difusores de auto</v>
+        <v>Difusores de varillas</v>
       </c>
       <c r="D13" t="str">
         <v>Relajantes</v>
@@ -11039,7 +11060,7 @@
         <v>Acondicionador-7</v>
       </c>
       <c r="C14" t="str">
-        <v>Difusor Wax Melt</v>
+        <v>Difusores de auto</v>
       </c>
       <c r="D14" t="str">
         <v>Sweetness Lavander</v>
@@ -11057,7 +11078,7 @@
         <v>Tónico para el cabello-8</v>
       </c>
       <c r="C15" t="str">
-        <v>Bruma</v>
+        <v>Difusor Wax Melt</v>
       </c>
       <c r="D15" t="str">
         <v>Orange Cold Brew</v>
@@ -11074,7 +11095,7 @@
         <v>Jabones corporales-9</v>
       </c>
       <c r="C16" t="str">
-        <v>Difusor + Wax Melt</v>
+        <v>Bruma</v>
       </c>
       <c r="D16" t="str">
         <v>Verdant Mint</v>
@@ -11085,7 +11106,7 @@
         <v>Velas aromáticas-17</v>
       </c>
       <c r="C17" t="str">
-        <v>Composición de velas</v>
+        <v>Difusor + Wax Melt</v>
       </c>
       <c r="D17" t="str">
         <v>Patchouli</v>
@@ -11099,7 +11120,7 @@
         <v>Difusores-18</v>
       </c>
       <c r="C18" t="str">
-        <v>Velas esculturales</v>
+        <v>Composición de velas</v>
       </c>
       <c r="D18" t="str">
         <v>Rosemary</v>
@@ -11111,7 +11132,7 @@
         <v>Sets-19</v>
       </c>
       <c r="C19" t="str">
-        <v>Arreglos florales</v>
+        <v>Velas esculturales</v>
       </c>
       <c r="D19" t="str">
         <v>Palo Santo</v>
@@ -11123,6 +11144,9 @@
     <row r="20" spans="2:16">
       <c r="B20" t="str">
         <v>Wax Melt-20</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Arreglos florales</v>
       </c>
       <c r="D20" t="str">
         <v>Sandalwood</v>
@@ -11595,10 +11619,10 @@
   <sheetData>
     <row r="2" spans="1:2" ht="15" thickBot="1"/>
     <row r="3" spans="1:2">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="52"/>
+      <c r="B3" s="56"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="7" t="s">

</xml_diff>